<commit_message>
Etapa 1: muros del perímetro hasta la altura final del 1er nivel (+2.30)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDAvj83gCUU9yQbmQvUtv6
</commit_message>
<xml_diff>
--- a/metrados/Etapa1_Cotizacion_CLIENTE.xlsx
+++ b/metrados/Etapa1_Cotizacion_CLIENTE.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -115,13 +115,6 @@
       <color rgb="FFC00000"/>
       <sz val="8"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="0"/>
-      <color rgb="00000000"/>
-      <sz val="9"/>
-    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -332,7 +325,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -347,7 +340,7 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="4" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -362,7 +355,7 @@
     <xf numFmtId="4" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="4" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="165" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -374,7 +367,7 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -662,7 +655,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -692,10 +684,10 @@
         </is>
       </c>
       <c r="B5" s="41" t="n">
-        <v>52798.19</v>
+        <v>53330.89</v>
       </c>
       <c r="C5" s="42" t="n">
-        <v>0.580909432680188</v>
+        <v>0.580010255667419</v>
       </c>
       <c r="D5" s="40" t="inlineStr">
         <is>
@@ -713,7 +705,7 @@
         <v>4715</v>
       </c>
       <c r="C6" s="42" t="n">
-        <v>0.051876550599312</v>
+        <v>0.051278880878828</v>
       </c>
       <c r="D6" s="40" t="inlineStr">
         <is>
@@ -728,10 +720,10 @@
         </is>
       </c>
       <c r="B7" s="41" t="n">
-        <v>30500</v>
+        <v>31000</v>
       </c>
       <c r="C7" s="42" t="n">
-        <v>0.335574717556525</v>
+        <v>0.337146406626441</v>
       </c>
       <c r="D7" s="40" t="inlineStr">
         <is>
@@ -746,10 +738,10 @@
         </is>
       </c>
       <c r="B8" s="44" t="n">
-        <v>88013.19</v>
+        <v>89045.89</v>
       </c>
       <c r="C8" s="42" t="n">
-        <v>0.968360700836025</v>
+        <v>0.968435543172688</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="36">
@@ -759,10 +751,10 @@
         </is>
       </c>
       <c r="B9" s="41" t="n">
-        <v>2875.6595</v>
+        <v>2902.2945</v>
       </c>
       <c r="C9" s="42" t="n">
-        <v>0.031639299163975</v>
+        <v>0.0315644568273123</v>
       </c>
       <c r="D9" s="40" t="inlineStr">
         <is>
@@ -777,7 +769,7 @@
         </is>
       </c>
       <c r="B10" s="44" t="n">
-        <v>90888.8495</v>
+        <v>91948.1845</v>
       </c>
       <c r="C10" s="42" t="n">
         <v>1</v>
@@ -795,7 +787,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="36">
       <c r="A13" s="45" t="inlineStr">
         <is>
@@ -828,7 +819,7 @@
         </is>
       </c>
       <c r="B15" s="41" t="n">
-        <v>4575</v>
+        <v>4650</v>
       </c>
       <c r="C15" s="46" t="n">
         <v>0.15</v>
@@ -841,7 +832,7 @@
         </is>
       </c>
       <c r="B16" s="41" t="n">
-        <v>9150</v>
+        <v>9300</v>
       </c>
       <c r="C16" s="46" t="n">
         <v>0.3</v>
@@ -854,7 +845,7 @@
         </is>
       </c>
       <c r="B17" s="41" t="n">
-        <v>3660</v>
+        <v>3720</v>
       </c>
       <c r="C17" s="46" t="n">
         <v>0.12</v>
@@ -867,7 +858,7 @@
         </is>
       </c>
       <c r="B18" s="41" t="n">
-        <v>7015</v>
+        <v>7130</v>
       </c>
       <c r="C18" s="46" t="n">
         <v>0.23</v>
@@ -880,7 +871,7 @@
         </is>
       </c>
       <c r="B19" s="41" t="n">
-        <v>6100</v>
+        <v>6200</v>
       </c>
       <c r="C19" s="46" t="n">
         <v>0.2</v>
@@ -893,13 +884,12 @@
         </is>
       </c>
       <c r="B20" s="44" t="n">
-        <v>30500</v>
+        <v>31000</v>
       </c>
       <c r="C20" s="47" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="21"/>
     <row r="22" ht="15" customHeight="1" s="36">
       <c r="A22" s="48" t="inlineStr">
         <is>
@@ -966,7 +956,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -1810,64 +1799,64 @@
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="36">
-      <c r="A34" s="40" t="inlineStr">
+      <c r="A34" s="54" t="inlineStr">
         <is>
           <t>05.02</t>
         </is>
       </c>
-      <c r="B34" s="40" t="inlineStr">
-        <is>
-          <t>Muro perímetro vivienda hasta +2.00 (con junta)</t>
-        </is>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
+      <c r="B34" s="54" t="inlineStr">
+        <is>
+          <t>Muro perímetro vivienda hasta +2.30 (altura final del 1er nivel, con junta)</t>
+        </is>
+      </c>
+      <c r="C34" s="54" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D34" s="41" t="n">
+      <c r="D34" s="55" t="n">
         <v>57.1</v>
       </c>
-      <c r="E34" s="51" t="n">
-        <v>57.1</v>
-      </c>
-      <c r="F34" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="53" t="inlineStr">
-        <is>
-          <t>31.7 m × 1.80</t>
+      <c r="E34" s="56" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="F34" s="57" t="n">
+        <v>9.499999999999989</v>
+      </c>
+      <c r="G34" s="58" t="inlineStr">
+        <is>
+          <t>31.7 m × 2.10 (de +0.20 a +2.30, fondo de viga). E-10 paraba en +2.00</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="36">
-      <c r="A35" s="40" t="inlineStr">
+      <c r="A35" s="54" t="inlineStr">
         <is>
           <t>05.03</t>
         </is>
       </c>
-      <c r="B35" s="40" t="inlineStr">
+      <c r="B35" s="54" t="inlineStr">
         <is>
           <t>Junta con tecnopor 1"</t>
         </is>
       </c>
-      <c r="C35" s="40" t="inlineStr">
+      <c r="C35" s="54" t="inlineStr">
         <is>
           <t>ml</t>
         </is>
       </c>
-      <c r="D35" s="41" t="n">
+      <c r="D35" s="55" t="n">
         <v>42</v>
       </c>
-      <c r="E35" s="51" t="n">
-        <v>42</v>
-      </c>
-      <c r="F35" s="52" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="53" t="inlineStr">
-        <is>
-          <t>Juntas muro-columna × 1.80 + cerco</t>
+      <c r="E35" s="56" t="n">
+        <v>48</v>
+      </c>
+      <c r="F35" s="57" t="n">
+        <v>6</v>
+      </c>
+      <c r="G35" s="58" t="inlineStr">
+        <is>
+          <t>E-10 42.0 + 20 juntas muro-columna × 0.30 adicionales</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1927,6 @@
       </c>
       <c r="G38" s="53" t="n"/>
     </row>
-    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="36">
       <c r="A40" s="59" t="inlineStr">
         <is>
@@ -1998,7 +1986,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -2189,17 +2176,17 @@
         </is>
       </c>
       <c r="D11" s="60" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E11" s="41" t="n">
         <v>28.6</v>
       </c>
       <c r="F11" s="41" t="n">
-        <v>1687.4</v>
+        <v>1744.6</v>
       </c>
       <c r="G11" s="40" t="inlineStr">
         <is>
-          <t>Solado 17 + ciclópeo 7 + sobrecim. 11 + solera 4 + mortero 20</t>
+          <t>Solado 17 + ciclópeo 7 + sobrecim. 11 + solera 4 + mortero 22</t>
         </is>
       </c>
     </row>
@@ -2247,17 +2234,17 @@
         </is>
       </c>
       <c r="D13" s="60" t="n">
-        <v>2.7</v>
+        <v>3</v>
       </c>
       <c r="E13" s="41" t="n">
         <v>65</v>
       </c>
       <c r="F13" s="41" t="n">
-        <v>175.5</v>
+        <v>195</v>
       </c>
       <c r="G13" s="40" t="inlineStr">
         <is>
-          <t>0.2 + 87 m² × 0.028</t>
+          <t>0.2 + 96.6 m² × 0.028</t>
         </is>
       </c>
     </row>
@@ -2609,17 +2596,17 @@
         </is>
       </c>
       <c r="D27" s="60" t="n">
-        <v>3560</v>
+        <v>3960</v>
       </c>
       <c r="E27" s="41" t="n">
         <v>1.14</v>
       </c>
       <c r="F27" s="41" t="n">
-        <v>4058.4</v>
+        <v>4514.4</v>
       </c>
       <c r="G27" s="40" t="inlineStr">
         <is>
-          <t>86.9 m² × 39 × 1.05</t>
+          <t>96.6 m² × 39 × 1.05</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2664,7 @@
       </c>
       <c r="G29" s="40" t="inlineStr">
         <is>
-          <t>12 m² ÷ 2.88</t>
+          <t>≈ 13.5 m² ÷ 2.88</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2729,7 @@
         </is>
       </c>
       <c r="F32" s="44" t="n">
-        <v>52798.19</v>
+        <v>53330.89</v>
       </c>
     </row>
   </sheetData>
@@ -2780,7 +2767,6 @@
     <row r="2" ht="15" customHeight="1" s="36">
       <c r="A2" s="38" t="n"/>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -3035,7 +3021,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -3683,13 +3668,13 @@
         </is>
       </c>
       <c r="D28" s="41" t="n">
-        <v>57.1</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="E28" s="51" t="n">
         <v>35</v>
       </c>
       <c r="F28" s="41" t="n">
-        <v>1998.5</v>
+        <v>2331</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="36">
@@ -3709,13 +3694,13 @@
         </is>
       </c>
       <c r="D29" s="41" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E29" s="51" t="n">
         <v>8</v>
       </c>
       <c r="F29" s="41" t="n">
-        <v>336</v>
+        <v>384</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="36">
@@ -3798,7 +3783,7 @@
         </is>
       </c>
       <c r="F33" s="44" t="n">
-        <v>30357.8</v>
+        <v>30738.3</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="36">
@@ -3808,7 +3793,7 @@
         </is>
       </c>
       <c r="F34" s="63" t="n">
-        <v>30500</v>
+        <v>31000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Etapa 1: VE conectadas a zapatas (-1.50) y sistema mixto con albañilería confinada en linderos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDAvj83gCUU9yQbmQvUtv6
</commit_message>
<xml_diff>
--- a/metrados/Etapa1_Cotizacion_CLIENTE.xlsx
+++ b/metrados/Etapa1_Cotizacion_CLIENTE.xlsx
@@ -691,10 +691,10 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>54431.49</v>
+        <v>53866.39</v>
       </c>
       <c r="C5" s="44" t="n">
-        <v>0.554835612431767</v>
+        <v>0.551644314127364</v>
       </c>
       <c r="D5" s="42" t="inlineStr">
         <is>
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="B6" s="43" t="n">
-        <v>4715</v>
+        <v>4845</v>
       </c>
       <c r="C6" s="44" t="n">
-        <v>0.048061332008655</v>
+        <v>0.0496175203489055</v>
       </c>
       <c r="D6" s="42" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         <v>36000</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>0.366958208337557</v>
+        <v>0.368675073799917</v>
       </c>
       <c r="D7" s="42" t="inlineStr">
         <is>
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="B8" s="46" t="n">
-        <v>95146.49000000001</v>
+        <v>94711.39</v>
       </c>
       <c r="C8" s="44" t="n">
-        <v>0.969855152777979</v>
+        <v>0.9699369082761869</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="38">
@@ -758,10 +758,10 @@
         </is>
       </c>
       <c r="B9" s="43" t="n">
-        <v>2957.3245</v>
+        <v>2935.5695</v>
       </c>
       <c r="C9" s="44" t="n">
-        <v>0.0301448472220211</v>
+        <v>0.0300630917238135</v>
       </c>
       <c r="D9" s="42" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="B10" s="46" t="n">
-        <v>98103.81449999999</v>
+        <v>97646.9595</v>
       </c>
       <c r="C10" s="44" t="n">
         <v>1</v>
@@ -921,7 +921,7 @@
     <row r="25" ht="15" customHeight="1" s="38">
       <c r="A25" s="50" t="inlineStr">
         <is>
-          <t>Nivel de VE según E-10 (de -1.00 a -0.30 sobre tecnopor). Si se cambia, se ajusta concreto, encofrado y excavación.</t>
+          <t>VE de -1.50 a -0.80 conectadas a las zapatas. Sistema mixto: linderos A y C de albañilería confinada (muro endentado de KK portante antes del vaciado de columnas).</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="37" min="1" max="1"/>
@@ -959,7 +959,7 @@
     <row r="2" ht="15" customHeight="1" s="38">
       <c r="A2" s="40" t="inlineStr">
         <is>
-          <t>Revisión del cuadro E-10 contra E-01, E-02/E-03, E-04. Filas en naranja = corregidas. VE de -1.00 a -0.30 sobre tecnopor (zanja de 1.10 de E-10).</t>
+          <t>Revisión del cuadro E-10 contra E-01, E-02/E-03, E-04. Filas en naranja = corregidas. VE de -1.50 a -0.80 conectadas a las zapatas (tecnopor debajo entre zapatas). Sistema mixto: albañilería confinada en linderos A y C.</t>
         </is>
       </c>
     </row>
@@ -1119,34 +1119,34 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="38">
-      <c r="A10" s="42" t="inlineStr">
+    <row r="10" ht="22.35" customHeight="1" s="38">
+      <c r="A10" s="56" t="inlineStr">
         <is>
           <t>02.02</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="56" t="inlineStr">
         <is>
           <t>Excavación zanjas VE / VC (retroexcavadora)</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="56" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D10" s="43" t="n">
+      <c r="D10" s="57" t="n">
         <v>24.3</v>
       </c>
-      <c r="E10" s="53" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="F10" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" s="55" t="inlineStr">
-        <is>
-          <t>VE 0.70×1.10×24.53 m = 18.9; VC 0.55×1.50×6.56 m = 5.4</t>
+      <c r="E10" s="58" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="F10" s="59" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G10" s="60" t="inlineStr">
+        <is>
+          <t>VE ahora con fondo -1.50 + tecnopor: 0.70×1.60×24.53 = 27.5; VC 0.55×1.50×6.56 = 5.4. (El modelo, descontando el sobreancho de pozos, da 28.3)</t>
         </is>
       </c>
     </row>
@@ -1201,14 +1201,14 @@
         <v>79.40000000000001</v>
       </c>
       <c r="E12" s="58" t="n">
-        <v>59.3</v>
+        <v>70.5</v>
       </c>
       <c r="F12" s="59" t="n">
-        <v>-20.1</v>
+        <v>-8.900000000000009</v>
       </c>
       <c r="G12" s="60" t="inlineStr">
         <is>
-          <t>Vivienda: 111.4 excav. - 44.9 enterrado (incl. sobrecimiento bajo -0.20) - 14.5 (capa superior 0.20) = 52.0; cerco 7.3. E-10 79.4 NO CABE en la excavación</t>
+          <t>Vivienda: excavación bajo -0.20 = 104.9 - enterrado 41.7 (solado, zapatas, VE, VC, tecnopor, columnas, sobrecimiento) = 63.2; cerco 7.3</t>
         </is>
       </c>
     </row>
@@ -1232,14 +1232,14 @@
         <v>53.5</v>
       </c>
       <c r="E13" s="58" t="n">
-        <v>81.7</v>
+        <v>78.5</v>
       </c>
       <c r="F13" s="59" t="n">
-        <v>28.2</v>
+        <v>25</v>
       </c>
       <c r="G13" s="60" t="inlineStr">
         <is>
-          <t>(124.7 - 59.3) × 1.25. E-10 sale bajo porque su relleno está inflado</t>
+          <t>(133.3 - 70.5) × 1.25</t>
         </is>
       </c>
     </row>
@@ -1338,14 +1338,14 @@
         <v>2.7</v>
       </c>
       <c r="E17" s="58" t="n">
-        <v>4.29</v>
+        <v>5.85</v>
       </c>
       <c r="F17" s="59" t="n">
-        <v>1.59</v>
+        <v>3.15</v>
       </c>
       <c r="G17" s="60" t="inlineStr">
         <is>
-          <t>Debe arrancar desde la viga, no desde -0.20: sobre VE (top -0.30) h = 0.50 → 20.98 m; sobre VC de ejes A y C (top -1.10) h ≈ 1.25 → 10.72 m; cerco h = 0.40 → 11.78 m</t>
+          <t>Arranca desde la viga: sobre VE (top -0.80) h = 1.00 → 20.98 m; sobre VC de ejes A y C (top -1.10 / zapata -1.00) h 1.20-1.30 → 10.72 m; cerco h = 0.40 → 11.78 m (medido en el modelo)</t>
         </is>
       </c>
     </row>
@@ -1369,14 +1369,14 @@
         <v>35.4</v>
       </c>
       <c r="E18" s="58" t="n">
-        <v>57.2</v>
+        <v>78</v>
       </c>
       <c r="F18" s="59" t="n">
-        <v>21.8</v>
+        <v>42.6</v>
       </c>
       <c r="G18" s="60" t="inlineStr">
         <is>
-          <t>2 × (0.50 × 20.98 + 1.25 × 10.72 + 0.40 × 11.78)</t>
+          <t>2 × (1.00 × 20.98 + 1.25 × 10.72 + 0.40 × 11.78)</t>
         </is>
       </c>
     </row>
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B21" s="56" t="inlineStr">
         <is>
-          <t>Vigas de equilibrio VE 0.30×0.70</t>
+          <t>Vigas de equilibrio VE 0.30×0.70 (de -1.50 a -0.80)</t>
         </is>
       </c>
       <c r="C21" s="56" t="inlineStr">
@@ -1444,14 +1444,14 @@
         <v>5.2</v>
       </c>
       <c r="E21" s="58" t="n">
-        <v>11.65</v>
+        <v>7.01</v>
       </c>
       <c r="F21" s="59" t="n">
-        <v>6.45</v>
+        <v>1.81</v>
       </c>
       <c r="G21" s="60" t="inlineStr">
         <is>
-          <t>E-10 solo mide 24.5 m entre zapatas. Con VE de -1.00 a -0.30 la viga va ENCIMA de la zapata: también se vacía el tramo sobre zapata (30.95 m). 0.21 × 55.47</t>
+          <t>Entre zapatas 0.30×0.70×24.53 = 5.15 + sobre zapata solo lo que sobresale (-1.00 a -0.80) 0.30×0.20×30.95 = 1.86</t>
         </is>
       </c>
     </row>
@@ -1475,14 +1475,14 @@
         <v>34.4</v>
       </c>
       <c r="E22" s="58" t="n">
-        <v>77.7</v>
+        <v>46.7</v>
       </c>
       <c r="F22" s="59" t="n">
-        <v>43.3</v>
+        <v>12.3</v>
       </c>
       <c r="G22" s="60" t="inlineStr">
         <is>
-          <t>2 × 0.70 × 55.47 (también sobre la zapata)</t>
+          <t>2 × 0.70 × 24.53 + 2 × 0.20 × 30.95</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="B23" s="42" t="inlineStr">
         <is>
-          <t>Tecnopor e = 0.10 bajo VE (solo entre zapatas)</t>
+          <t>Tecnopor e = 0.10 bajo VE (solo entre zapatas, de -1.60 a -1.50)</t>
         </is>
       </c>
       <c r="C23" s="42" t="inlineStr">
@@ -1599,45 +1599,45 @@
         <v>8.199999999999999</v>
       </c>
       <c r="E26" s="53" t="n">
-        <v>8.220000000000001</v>
+        <v>8.32</v>
       </c>
       <c r="F26" s="54" t="n">
-        <v>0.0200000000000014</v>
+        <v>0.120000000000001</v>
       </c>
       <c r="G26" s="55" t="inlineStr">
         <is>
-          <t>2.49 m² × 3.30</t>
+          <t>2.49 m² × 3.30 = 8.22 + 0.10 de concreto que entra en los dientes del muro</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="38">
-      <c r="A27" s="42" t="inlineStr">
+      <c r="A27" s="56" t="inlineStr">
         <is>
           <t>04.07</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B27" s="56" t="inlineStr">
         <is>
           <t>Encofrado columnas 1er piso</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C27" s="56" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D27" s="43" t="n">
+      <c r="D27" s="57" t="n">
         <v>83.5</v>
       </c>
-      <c r="E27" s="53" t="n">
-        <v>83.5</v>
-      </c>
-      <c r="F27" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="55" t="inlineStr">
-        <is>
-          <t>Perímetros 25.3 m × 3.30</t>
+      <c r="E27" s="58" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="F27" s="59" t="n">
+        <v>-4.40000000000001</v>
+      </c>
+      <c r="G27" s="60" t="inlineStr">
+        <is>
+          <t>25.3 m × 3.30 = 83.5 - 16 caras contra muro endentado (0.13 × 2.10) = 4.4</t>
         </is>
       </c>
     </row>
@@ -1808,12 +1808,12 @@
     <row r="34" ht="15" customHeight="1" s="38">
       <c r="A34" s="56" t="inlineStr">
         <is>
-          <t>05.02</t>
+          <t>05.02a</t>
         </is>
       </c>
       <c r="B34" s="56" t="inlineStr">
         <is>
-          <t>Muro perímetro vivienda hasta +2.30 (altura final del 1er nivel, con junta)</t>
+          <t>Muro portante linderos A y C - KK PORTANTE endentado (albañilería confinada)</t>
         </is>
       </c>
       <c r="C34" s="56" t="inlineStr">
@@ -1825,138 +1825,169 @@
         <v>57.1</v>
       </c>
       <c r="E34" s="58" t="n">
-        <v>66.59999999999999</v>
+        <v>52.5</v>
       </c>
       <c r="F34" s="59" t="n">
-        <v>9.499999999999989</v>
+        <v>-4.6</v>
       </c>
       <c r="G34" s="60" t="inlineStr">
         <is>
-          <t>31.7 m × 2.10 (de +0.20 a +2.30, fondo de viga). E-10 paraba en +2.00</t>
+          <t>2 × 12.50 × 2.10 (de +0.20 a +2.30). Se levanta ANTES de vaciar las columnas</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="38">
       <c r="A35" s="56" t="inlineStr">
         <is>
+          <t>05.02b</t>
+        </is>
+      </c>
+      <c r="B35" s="56" t="inlineStr">
+        <is>
+          <t>Muro fondo eje 5 - tabique KK 18 huecos con junta</t>
+        </is>
+      </c>
+      <c r="C35" s="56" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D35" s="57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="58" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="F35" s="59" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="G35" s="60" t="inlineStr">
+        <is>
+          <t>6.70 × 2.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1" s="38">
+      <c r="A36" s="56" t="inlineStr">
+        <is>
           <t>05.03</t>
         </is>
       </c>
-      <c r="B35" s="56" t="inlineStr">
-        <is>
-          <t>Junta con tecnopor 1"</t>
-        </is>
-      </c>
-      <c r="C35" s="56" t="inlineStr">
+      <c r="B36" s="56" t="inlineStr">
+        <is>
+          <t>Junta con tecnopor 1" (solo fondo y encuentro cerco-vivienda)</t>
+        </is>
+      </c>
+      <c r="C36" s="56" t="inlineStr">
         <is>
           <t>ml</t>
         </is>
       </c>
-      <c r="D35" s="57" t="n">
+      <c r="D36" s="57" t="n">
         <v>42</v>
       </c>
-      <c r="E35" s="58" t="n">
-        <v>48</v>
-      </c>
-      <c r="F35" s="59" t="n">
-        <v>6</v>
-      </c>
-      <c r="G35" s="60" t="inlineStr">
-        <is>
-          <t>E-10 42.0 + 20 juntas muro-columna × 0.30 adicionales</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="38">
-      <c r="A36" s="51" t="inlineStr">
+      <c r="E36" s="58" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="F36" s="59" t="n">
+        <v>-28.4</v>
+      </c>
+      <c r="G36" s="60" t="inlineStr">
+        <is>
+          <t>Linderos ya no llevan junta (muro endentado). Fondo 4 × 2.10 + cerco-vivienda 2 × 2.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="38">
+      <c r="A37" s="51" t="inlineStr">
         <is>
           <t>06  VARIOS</t>
         </is>
       </c>
-      <c r="B36" s="52" t="n"/>
-      <c r="C36" s="52" t="n"/>
-      <c r="D36" s="52" t="n"/>
-      <c r="E36" s="52" t="n"/>
-      <c r="F36" s="52" t="n"/>
-      <c r="G36" s="52" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="38">
-      <c r="A37" s="42" t="inlineStr">
-        <is>
-          <t>06.01</t>
-        </is>
-      </c>
-      <c r="B37" s="42" t="inlineStr">
-        <is>
-          <t>Curado de concreto</t>
-        </is>
-      </c>
-      <c r="C37" s="42" t="inlineStr">
-        <is>
-          <t>glb</t>
-        </is>
-      </c>
-      <c r="D37" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="E37" s="53" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="55" t="n"/>
+      <c r="B37" s="52" t="n"/>
+      <c r="C37" s="52" t="n"/>
+      <c r="D37" s="52" t="n"/>
+      <c r="E37" s="52" t="n"/>
+      <c r="F37" s="52" t="n"/>
+      <c r="G37" s="52" t="n"/>
     </row>
     <row r="38" ht="15" customHeight="1" s="38">
       <c r="A38" s="42" t="inlineStr">
         <is>
-          <t>06.02</t>
+          <t>06.01</t>
         </is>
       </c>
       <c r="B38" s="42" t="inlineStr">
         <is>
-          <t>Ensayo de probetas</t>
+          <t>Curado de concreto</t>
         </is>
       </c>
       <c r="C38" s="42" t="inlineStr">
         <is>
-          <t>juego</t>
+          <t>glb</t>
         </is>
       </c>
       <c r="D38" s="43" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E38" s="53" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F38" s="54" t="n">
         <v>0</v>
       </c>
       <c r="G38" s="55" t="n"/>
     </row>
-    <row r="40" ht="15" customHeight="1" s="38">
-      <c r="A40" s="61" t="inlineStr">
-        <is>
-          <t>IMPORTANTE - NIVEL DE LA VE: E-10 usa VE de -1.00 a -0.30 (zanja de 1.10 y tecnopor debajo). Si la VE va con fondo a -1.50 (al mismo nivel que la zapata),</t>
-        </is>
-      </c>
+    <row r="39" ht="15" customHeight="1" s="38">
+      <c r="A39" s="42" t="inlineStr">
+        <is>
+          <t>06.02</t>
+        </is>
+      </c>
+      <c r="B39" s="42" t="inlineStr">
+        <is>
+          <t>Ensayo de probetas</t>
+        </is>
+      </c>
+      <c r="C39" s="42" t="inlineStr">
+        <is>
+          <t>juego</t>
+        </is>
+      </c>
+      <c r="D39" s="43" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="F39" s="54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="55" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1" s="38">
       <c r="A41" s="61" t="inlineStr">
         <is>
-          <t>el concreto de VE baja a 7.0 m³ y el encofrado a 46.7 m², pero la zanja de VE sube a 1.60 de profundidad (27.5 m³). Definir antes de comprar.</t>
+          <t>CAMBIOS DE OBRA: VE de -1.50 a -0.80 conectadas a las zapatas (tecnopor 0.10 bajo VE entre zapatas, excavación a -1.60).</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="38">
       <c r="A42" s="61" t="inlineStr">
         <is>
-          <t>Acero de columnas 1er piso: 2,646 kg (E-10) verificado (barras Ø5/8" de 6.00 m de arranque + estribos Ø1/2" 1,342 kg + montaje 3/8" 38 kg).</t>
+          <t>Sistema mixto: linderos A y C de albañilería confinada (KK portante con ≤30% vacíos, E.070), muro endentado y luego vaciado de columnas.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="38">
       <c r="A43" s="61" t="inlineStr">
+        <is>
+          <t>Acero de columnas 1er piso: 2,646 kg (E-10) verificado (barras Ø5/8" de 6.00 m de arranque + estribos Ø1/2" 1,342 kg + montaje 3/8" 38 kg).</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="15" customHeight="1" s="38">
+      <c r="A44" s="61" t="inlineStr">
         <is>
           <t>Diferencias menores a favor (no se cambian): zanjas de VE medidas sin descontar el sobreancho de los pozos (~2.5 m³ de más); encofrado de columnas sin descontar las caras donde llega la VE (~6.7 m²).</t>
         </is>
@@ -1975,7 +2006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="37" min="1" max="1"/>
@@ -2065,17 +2096,17 @@
         </is>
       </c>
       <c r="D6" s="62" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E6" s="43" t="n">
         <v>320</v>
       </c>
       <c r="F6" s="43" t="n">
-        <v>13440</v>
+        <v>11840</v>
       </c>
       <c r="G6" s="42" t="inlineStr">
         <is>
-          <t>(23.39 + 11.65 + 0.66 + 1.36 + 1.18) × 1.04 = 39.8 + 2.0 por sobreexcavación de la retro → 42.0</t>
+          <t>(23.39 + 7.01 + 0.66 + 1.36 + 1.18) × 1.04 = 34.9 + 2.0 por sobreexcavación de la retro → 37.0</t>
         </is>
       </c>
     </row>
@@ -2094,13 +2125,13 @@
         </is>
       </c>
       <c r="D7" s="62" t="n">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="E7" s="43" t="n">
         <v>38</v>
       </c>
       <c r="F7" s="43" t="n">
-        <v>1596</v>
+        <v>1406</v>
       </c>
       <c r="G7" s="42" t="n"/>
     </row>
@@ -2190,17 +2221,17 @@
         </is>
       </c>
       <c r="D11" s="62" t="n">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E11" s="43" t="n">
         <v>28.6</v>
       </c>
       <c r="F11" s="43" t="n">
-        <v>1916.2</v>
+        <v>2087.8</v>
       </c>
       <c r="G11" s="42" t="inlineStr">
         <is>
-          <t>Solado 17 + ciclópeo 7 + sobrecim. 17 + solera 4 + mortero 22</t>
+          <t>Solado 17 + ciclópeo 7 + sobrecim. 23 + solera 4 + mortero 22</t>
         </is>
       </c>
     </row>
@@ -2219,17 +2250,17 @@
         </is>
       </c>
       <c r="D12" s="62" t="n">
-        <v>11</v>
+        <v>12.4</v>
       </c>
       <c r="E12" s="43" t="n">
         <v>60</v>
       </c>
       <c r="F12" s="43" t="n">
-        <v>660</v>
+        <v>744</v>
       </c>
       <c r="G12" s="42" t="inlineStr">
         <is>
-          <t>5.4 + 1.9 + 3.7</t>
+          <t>5.4 + 1.9 + 5.1</t>
         </is>
       </c>
     </row>
@@ -2327,13 +2358,13 @@
         </is>
       </c>
       <c r="D16" s="62" t="n">
-        <v>1.7</v>
+        <v>2.3</v>
       </c>
       <c r="E16" s="43" t="n">
         <v>50</v>
       </c>
       <c r="F16" s="43" t="n">
-        <v>85</v>
+        <v>115</v>
       </c>
       <c r="G16" s="42" t="n"/>
     </row>
@@ -2552,17 +2583,17 @@
         </is>
       </c>
       <c r="D25" s="62" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E25" s="43" t="n">
         <v>6.5</v>
       </c>
       <c r="F25" s="43" t="n">
-        <v>403</v>
+        <v>377</v>
       </c>
       <c r="G25" s="42" t="inlineStr">
         <is>
-          <t>0.25 kg/m² × 246 m²</t>
+          <t>0.25 kg/m² × 231 m²</t>
         </is>
       </c>
     </row>
@@ -2581,17 +2612,17 @@
         </is>
       </c>
       <c r="D26" s="62" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E26" s="43" t="n">
         <v>7.5</v>
       </c>
       <c r="F26" s="43" t="n">
-        <v>277.5</v>
+        <v>262.5</v>
       </c>
       <c r="G26" s="42" t="inlineStr">
         <is>
-          <t>0.15 kg/m² × 246 m²</t>
+          <t>0.15 kg/m² × 231 m²</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2632,7 @@
       </c>
       <c r="B27" s="42" t="inlineStr">
         <is>
-          <t>Ladrillo KK 18 huecos (+5%)</t>
+          <t>Ladrillo KK PORTANTE - linderos A y C (+5%)</t>
         </is>
       </c>
       <c r="C27" s="42" t="inlineStr">
@@ -2610,17 +2641,17 @@
         </is>
       </c>
       <c r="D27" s="62" t="n">
-        <v>3960</v>
+        <v>2150</v>
       </c>
       <c r="E27" s="43" t="n">
-        <v>1.14</v>
+        <v>1.6</v>
       </c>
       <c r="F27" s="43" t="n">
-        <v>4514.4</v>
+        <v>3440</v>
       </c>
       <c r="G27" s="42" t="inlineStr">
         <is>
-          <t>96.6 m² × 39 × 1.05</t>
+          <t>52.5 m² × 39 × 1.05. Obligatorio en muro portante zona 4 (E.070)</t>
         </is>
       </c>
     </row>
@@ -2630,26 +2661,26 @@
       </c>
       <c r="B28" s="42" t="inlineStr">
         <is>
-          <t>Tecnopor 4" bajo VE</t>
+          <t>Ladrillo KK 18 huecos - fondo y cerco (+5%)</t>
         </is>
       </c>
       <c r="C28" s="42" t="inlineStr">
         <is>
-          <t>plancha</t>
+          <t>und</t>
         </is>
       </c>
       <c r="D28" s="62" t="n">
-        <v>3</v>
+        <v>1805</v>
       </c>
       <c r="E28" s="43" t="n">
-        <v>55</v>
+        <v>1.14</v>
       </c>
       <c r="F28" s="43" t="n">
-        <v>165</v>
+        <v>2057.7</v>
       </c>
       <c r="G28" s="42" t="inlineStr">
         <is>
-          <t>7.4 m² ÷ 2.88</t>
+          <t>(14.1 + 30.0) m² × 39 × 1.05</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2690,7 @@
       </c>
       <c r="B29" s="42" t="inlineStr">
         <is>
-          <t>Tecnopor 1" para juntas</t>
+          <t>Tecnopor 4" bajo VE</t>
         </is>
       </c>
       <c r="C29" s="42" t="inlineStr">
@@ -2668,17 +2699,17 @@
         </is>
       </c>
       <c r="D29" s="62" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E29" s="43" t="n">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="F29" s="43" t="n">
-        <v>80</v>
+        <v>165</v>
       </c>
       <c r="G29" s="42" t="inlineStr">
         <is>
-          <t>≈ 13.5 m² ÷ 2.88</t>
+          <t>7.4 m² ÷ 2.88</t>
         </is>
       </c>
     </row>
@@ -2688,26 +2719,26 @@
       </c>
       <c r="B30" s="42" t="inlineStr">
         <is>
-          <t>Epóxico para anclajes</t>
+          <t>Tecnopor 1" para juntas</t>
         </is>
       </c>
       <c r="C30" s="42" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>plancha</t>
         </is>
       </c>
       <c r="D30" s="62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E30" s="43" t="n">
-        <v>120</v>
+        <v>16</v>
       </c>
       <c r="F30" s="43" t="n">
-        <v>120</v>
+        <v>32</v>
       </c>
       <c r="G30" s="42" t="inlineStr">
         <is>
-          <t>8 anclajes</t>
+          <t>13.6 ml × 0.13 ≈ 1.8 m² + cortes</t>
         </is>
       </c>
     </row>
@@ -2717,33 +2748,62 @@
       </c>
       <c r="B31" s="42" t="inlineStr">
         <is>
+          <t>Epóxico para anclajes</t>
+        </is>
+      </c>
+      <c r="C31" s="42" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="D31" s="62" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="43" t="n">
+        <v>120</v>
+      </c>
+      <c r="F31" s="43" t="n">
+        <v>120</v>
+      </c>
+      <c r="G31" s="42" t="inlineStr">
+        <is>
+          <t>8 anclajes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="38">
+      <c r="A32" s="42" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" s="42" t="inlineStr">
+        <is>
           <t>Impermeabilizante asfáltico (sobrecimiento)</t>
         </is>
       </c>
-      <c r="C31" s="42" t="inlineStr">
+      <c r="C32" s="42" t="inlineStr">
         <is>
           <t>gal</t>
         </is>
       </c>
-      <c r="D31" s="62" t="n">
-        <v>3</v>
-      </c>
-      <c r="E31" s="43" t="n">
+      <c r="D32" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" s="43" t="n">
         <v>45</v>
       </c>
-      <c r="F31" s="43" t="n">
-        <v>135</v>
-      </c>
-      <c r="G31" s="42" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="38">
-      <c r="E32" s="45" t="inlineStr">
+      <c r="F32" s="43" t="n">
+        <v>180</v>
+      </c>
+      <c r="G32" s="42" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="38">
+      <c r="E33" s="45" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F32" s="46" t="n">
-        <v>54431.49</v>
+      <c r="F33" s="46" t="n">
+        <v>53866.39</v>
       </c>
     </row>
   </sheetData>
@@ -2843,7 +2903,7 @@
       </c>
       <c r="G5" s="42" t="inlineStr">
         <is>
-          <t>81.7 m³ suelto ÷ 18</t>
+          <t>78.5 m³ suelto ÷ 18</t>
         </is>
       </c>
     </row>
@@ -2862,17 +2922,17 @@
         </is>
       </c>
       <c r="D6" s="62" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6" s="43" t="n">
         <v>130</v>
       </c>
       <c r="F6" s="43" t="n">
-        <v>1040</v>
+        <v>1170</v>
       </c>
       <c r="G6" s="42" t="inlineStr">
         <is>
-          <t>59 m³ ÷ 8 m³/día</t>
+          <t>70.5 m³ ÷ 8 m³/día</t>
         </is>
       </c>
     </row>
@@ -2991,7 +3051,7 @@
         </is>
       </c>
       <c r="F11" s="46" t="n">
-        <v>4715</v>
+        <v>4845</v>
       </c>
     </row>
   </sheetData>
@@ -3007,7 +3067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="37" min="1" max="1"/>
@@ -3093,10 +3153,10 @@
         <v>170</v>
       </c>
       <c r="E5" s="43" t="n">
-        <v>2.3</v>
+        <v>2.28</v>
       </c>
       <c r="F5" s="43" t="n">
-        <v>391</v>
+        <v>387.6</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="38">
@@ -3119,10 +3179,10 @@
         <v>170</v>
       </c>
       <c r="E6" s="43" t="n">
-        <v>3.44</v>
+        <v>3.43</v>
       </c>
       <c r="F6" s="43" t="n">
-        <v>584.8</v>
+        <v>583.1</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="38">
@@ -3142,13 +3202,13 @@
         </is>
       </c>
       <c r="D7" s="43" t="n">
-        <v>111.4</v>
+        <v>120</v>
       </c>
       <c r="E7" s="43" t="n">
-        <v>36.74</v>
+        <v>36.55</v>
       </c>
       <c r="F7" s="43" t="n">
-        <v>4092.836</v>
+        <v>4386</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="38">
@@ -3171,10 +3231,10 @@
         <v>75.2</v>
       </c>
       <c r="E8" s="43" t="n">
-        <v>6.89</v>
+        <v>6.85</v>
       </c>
       <c r="F8" s="43" t="n">
-        <v>518.128</v>
+        <v>515.12</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="38">
@@ -3197,10 +3257,10 @@
         <v>13.3</v>
       </c>
       <c r="E9" s="43" t="n">
-        <v>51.67</v>
+        <v>51.39</v>
       </c>
       <c r="F9" s="43" t="n">
-        <v>687.211</v>
+        <v>683.487</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="38">
@@ -3220,13 +3280,13 @@
         </is>
       </c>
       <c r="D10" s="43" t="n">
-        <v>59.3</v>
+        <v>70.5</v>
       </c>
       <c r="E10" s="43" t="n">
-        <v>34.44</v>
+        <v>34.26</v>
       </c>
       <c r="F10" s="43" t="n">
-        <v>2042.292</v>
+        <v>2415.33</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="38">
@@ -3249,10 +3309,10 @@
         <v>50</v>
       </c>
       <c r="E11" s="43" t="n">
-        <v>17.22</v>
+        <v>17.13</v>
       </c>
       <c r="F11" s="43" t="n">
-        <v>861</v>
+        <v>856.5</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="38">
@@ -3275,10 +3335,10 @@
         <v>2.2</v>
       </c>
       <c r="E12" s="43" t="n">
-        <v>103.33</v>
+        <v>102.79</v>
       </c>
       <c r="F12" s="43" t="n">
-        <v>227.326</v>
+        <v>226.138</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="38">
@@ -3298,13 +3358,13 @@
         </is>
       </c>
       <c r="D13" s="43" t="n">
-        <v>4.29</v>
+        <v>5.85</v>
       </c>
       <c r="E13" s="43" t="n">
-        <v>137.78</v>
+        <v>137.05</v>
       </c>
       <c r="F13" s="43" t="n">
-        <v>591.0762</v>
+        <v>801.7424999999999</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="38">
@@ -3324,13 +3384,13 @@
         </is>
       </c>
       <c r="D14" s="43" t="n">
-        <v>57.2</v>
+        <v>78</v>
       </c>
       <c r="E14" s="43" t="n">
-        <v>25.26</v>
+        <v>25.13</v>
       </c>
       <c r="F14" s="43" t="n">
-        <v>1444.872</v>
+        <v>1960.14</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="38">
@@ -3402,13 +3462,13 @@
         </is>
       </c>
       <c r="D17" s="53" t="n">
-        <v>82.90000000000001</v>
+        <v>51.9</v>
       </c>
       <c r="E17" s="43" t="n">
-        <v>28.7</v>
+        <v>28.55</v>
       </c>
       <c r="F17" s="43" t="n">
-        <v>2379.23</v>
+        <v>1481.745</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="38">
@@ -3431,10 +3491,10 @@
         <v>7.4</v>
       </c>
       <c r="E18" s="43" t="n">
-        <v>5.74</v>
+        <v>5.71</v>
       </c>
       <c r="F18" s="43" t="n">
-        <v>42.476</v>
+        <v>42.254</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="38">
@@ -3445,7 +3505,7 @@
       </c>
       <c r="B19" s="42" t="inlineStr">
         <is>
-          <t>Vaciado y vibrado premezclado - cimentación (42 m³)</t>
+          <t>Vaciado y vibrado premezclado - cimentación (37 m³)</t>
         </is>
       </c>
       <c r="C19" s="42" t="inlineStr">
@@ -3454,13 +3514,13 @@
         </is>
       </c>
       <c r="D19" s="53" t="n">
-        <v>38.2</v>
+        <v>33.6</v>
       </c>
       <c r="E19" s="43" t="n">
-        <v>45.93</v>
+        <v>45.68</v>
       </c>
       <c r="F19" s="43" t="n">
-        <v>1754.526</v>
+        <v>1534.848</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="38">
@@ -3483,10 +3543,10 @@
         <v>2646</v>
       </c>
       <c r="E20" s="43" t="n">
-        <v>1.49</v>
+        <v>1.48</v>
       </c>
       <c r="F20" s="43" t="n">
-        <v>3942.54</v>
+        <v>3916.08</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="38">
@@ -3506,13 +3566,13 @@
         </is>
       </c>
       <c r="D21" s="43" t="n">
-        <v>83.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="E21" s="43" t="n">
-        <v>32.15</v>
+        <v>31.98</v>
       </c>
       <c r="F21" s="43" t="n">
-        <v>2684.525</v>
+        <v>2529.618</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="38">
@@ -3523,7 +3583,7 @@
       </c>
       <c r="B22" s="42" t="inlineStr">
         <is>
-          <t>Vaciado y vibrado premezclado - columnas + CA</t>
+          <t>Vaciado y vibrado premezclado - columnas + CA (contra muro endentado)</t>
         </is>
       </c>
       <c r="C22" s="42" t="inlineStr">
@@ -3532,13 +3592,13 @@
         </is>
       </c>
       <c r="D22" s="53" t="n">
-        <v>8.800000000000001</v>
+        <v>8.9</v>
       </c>
       <c r="E22" s="43" t="n">
-        <v>68.89</v>
+        <v>68.52</v>
       </c>
       <c r="F22" s="43" t="n">
-        <v>606.232</v>
+        <v>609.828</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="38">
@@ -3561,10 +3621,10 @@
         <v>304</v>
       </c>
       <c r="E23" s="43" t="n">
-        <v>1.38</v>
+        <v>1.37</v>
       </c>
       <c r="F23" s="43" t="n">
-        <v>419.52</v>
+        <v>416.48</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="38">
@@ -3587,10 +3647,10 @@
         <v>21.9</v>
       </c>
       <c r="E24" s="43" t="n">
-        <v>28.7</v>
+        <v>28.55</v>
       </c>
       <c r="F24" s="43" t="n">
-        <v>628.53</v>
+        <v>625.245</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="38">
@@ -3613,10 +3673,10 @@
         <v>0.37</v>
       </c>
       <c r="E25" s="43" t="n">
-        <v>137.78</v>
+        <v>137.05</v>
       </c>
       <c r="F25" s="43" t="n">
-        <v>50.9786</v>
+        <v>50.7085</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="38">
@@ -3639,10 +3699,10 @@
         <v>8</v>
       </c>
       <c r="E26" s="43" t="n">
-        <v>22.96</v>
+        <v>22.84</v>
       </c>
       <c r="F26" s="43" t="n">
-        <v>183.68</v>
+        <v>182.72</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="38">
@@ -3665,21 +3725,21 @@
         <v>29.8</v>
       </c>
       <c r="E27" s="43" t="n">
-        <v>40.19</v>
+        <v>39.97</v>
       </c>
       <c r="F27" s="43" t="n">
-        <v>1197.662</v>
+        <v>1191.106</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="38">
       <c r="A28" s="42" t="inlineStr">
         <is>
-          <t>05.02</t>
+          <t>05.02a</t>
         </is>
       </c>
       <c r="B28" s="42" t="inlineStr">
         <is>
-          <t>Muro KK de soga - perímetro vivienda</t>
+          <t>Muro portante KK endentado - linderos (albañilería confinada)</t>
         </is>
       </c>
       <c r="C28" s="42" t="inlineStr">
@@ -3688,131 +3748,157 @@
         </is>
       </c>
       <c r="D28" s="43" t="n">
-        <v>66.59999999999999</v>
+        <v>52.5</v>
       </c>
       <c r="E28" s="43" t="n">
-        <v>40.19</v>
+        <v>45.68</v>
       </c>
       <c r="F28" s="43" t="n">
-        <v>2676.654</v>
+        <v>2398.2</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="38">
       <c r="A29" s="42" t="inlineStr">
         <is>
-          <t>05.03</t>
+          <t>05.02b</t>
         </is>
       </c>
       <c r="B29" s="42" t="inlineStr">
         <is>
-          <t>Junta con tecnopor 1"</t>
+          <t>Muro KK de soga - fondo (tabique con junta)</t>
         </is>
       </c>
       <c r="C29" s="42" t="inlineStr">
         <is>
-          <t>ml</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="D29" s="43" t="n">
-        <v>48</v>
+        <v>14.1</v>
       </c>
       <c r="E29" s="43" t="n">
-        <v>9.19</v>
+        <v>39.97</v>
       </c>
       <c r="F29" s="43" t="n">
-        <v>441.12</v>
+        <v>563.577</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="38">
       <c r="A30" s="42" t="inlineStr">
         <is>
-          <t>06.01</t>
+          <t>05.03</t>
         </is>
       </c>
       <c r="B30" s="42" t="inlineStr">
         <is>
-          <t>Curado de concreto (riego diario)</t>
+          <t>Junta con tecnopor 1"</t>
         </is>
       </c>
       <c r="C30" s="42" t="inlineStr">
         <is>
-          <t>día</t>
-        </is>
-      </c>
-      <c r="D30" s="53" t="n">
-        <v>14</v>
+          <t>ml</t>
+        </is>
+      </c>
+      <c r="D30" s="43" t="n">
+        <v>13.6</v>
       </c>
       <c r="E30" s="43" t="n">
-        <v>45.93</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="F30" s="43" t="n">
-        <v>643.02</v>
+        <v>124.304</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="38">
       <c r="A31" s="42" t="inlineStr">
         <is>
+          <t>06.01</t>
+        </is>
+      </c>
+      <c r="B31" s="42" t="inlineStr">
+        <is>
+          <t>Curado de concreto (riego diario)</t>
+        </is>
+      </c>
+      <c r="C31" s="42" t="inlineStr">
+        <is>
+          <t>día</t>
+        </is>
+      </c>
+      <c r="D31" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="E31" s="43" t="n">
+        <v>45.68</v>
+      </c>
+      <c r="F31" s="43" t="n">
+        <v>639.52</v>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="38">
+      <c r="A32" s="42" t="inlineStr">
+        <is>
           <t>06.03</t>
         </is>
       </c>
-      <c r="B31" s="42" t="inlineStr">
+      <c r="B32" s="42" t="inlineStr">
         <is>
           <t>Limpieza final</t>
         </is>
       </c>
-      <c r="C31" s="42" t="inlineStr">
+      <c r="C32" s="42" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D31" s="53" t="n">
+      <c r="D32" s="53" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="43" t="n">
-        <v>344.45</v>
-      </c>
-      <c r="F31" s="43" t="n">
-        <v>344.45</v>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="38">
-      <c r="B32" s="42" t="inlineStr">
+      <c r="E32" s="43" t="n">
+        <v>342.62</v>
+      </c>
+      <c r="F32" s="43" t="n">
+        <v>342.62</v>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="38">
+      <c r="B33" s="42" t="inlineStr">
         <is>
           <t>Dirección técnica y residencia de obra</t>
         </is>
       </c>
-      <c r="C32" s="42" t="inlineStr">
+      <c r="C33" s="42" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D32" s="63" t="n">
+      <c r="D33" s="63" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="43" t="n">
-        <v>2870.38</v>
-      </c>
-      <c r="F32" s="43" t="n">
-        <v>2870.38</v>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="38">
-      <c r="E33" s="45" t="inlineStr">
+      <c r="E33" s="43" t="n">
+        <v>2855.17</v>
+      </c>
+      <c r="F33" s="43" t="n">
+        <v>2855.17</v>
+      </c>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="38">
+      <c r="E34" s="45" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F33" s="46" t="n">
-        <v>35985.2648</v>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="38">
-      <c r="E34" s="64" t="inlineStr">
+      <c r="F34" s="46" t="n">
+        <v>35998.381</v>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="38">
+      <c r="E35" s="64" t="inlineStr">
         <is>
           <t>A cotizar (redondeado)</t>
         </is>
       </c>
-      <c r="F34" s="65" t="n">
+      <c r="F35" s="65" t="n">
         <v>36000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Etapa 1: hoja interna Opción A (reducción de acero VE/VC) para decidir en campo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JDAvj83gCUU9yQbmQvUtv6
</commit_message>
<xml_diff>
--- a/metrados/Etapa1_Cotizacion_CLIENTE.xlsx
+++ b/metrados/Etapa1_Cotizacion_CLIENTE.xlsx
@@ -189,7 +189,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -299,6 +299,21 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="3" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -642,284 +657,284 @@
   <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="66" customWidth="1" style="37" min="1" max="1"/>
-    <col width="14" customWidth="1" style="37" min="2" max="2"/>
-    <col width="8" customWidth="1" style="37" min="3" max="3"/>
-    <col width="44" customWidth="1" style="37" min="4" max="4"/>
+    <col width="66" customWidth="1" style="42" min="1" max="1"/>
+    <col width="14" customWidth="1" style="42" min="2" max="2"/>
+    <col width="8" customWidth="1" style="42" min="3" max="3"/>
+    <col width="44" customWidth="1" style="42" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="38">
-      <c r="A1" s="39" t="inlineStr">
+    <row r="1" ht="16.15" customHeight="1" s="43">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>COTIZACIÓN ETAPA 1 - VIVIENDA UNIFAMILIAR, CHORRILLOS</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="38">
-      <c r="A2" s="40" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="43">
+      <c r="A2" s="45" t="inlineStr">
         <is>
           <t>Cimentación, columnas 1er piso hasta +2.30, cerco delantero y muros del perímetro (E-10). Precios Lima, octubre 2026.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" s="38">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="4" ht="31.5" customHeight="1" s="43">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>Monto (S/)</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Quién paga</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="38">
-      <c r="A5" s="42" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="43">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>A. Materiales</t>
         </is>
       </c>
-      <c r="B5" s="43" t="n">
+      <c r="B5" s="48" t="n">
         <v>53866.39</v>
       </c>
-      <c r="C5" s="44" t="n">
+      <c r="C5" s="49" t="n">
         <v>0.551644314127364</v>
       </c>
-      <c r="D5" s="42" t="inlineStr">
+      <c r="D5" s="47" t="inlineStr">
         <is>
           <t>Cliente - compra directa con boleta/factura</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="38">
-      <c r="A6" s="42" t="inlineStr">
+    <row r="6" ht="15" customHeight="1" s="43">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>B. Equipos y servicios (volquetes, apisonador, probetas, agua, flete)</t>
         </is>
       </c>
-      <c r="B6" s="43" t="n">
+      <c r="B6" s="48" t="n">
         <v>4845</v>
       </c>
-      <c r="C6" s="44" t="n">
+      <c r="C6" s="49" t="n">
         <v>0.0496175203489055</v>
       </c>
-      <c r="D6" s="42" t="inlineStr">
+      <c r="D6" s="47" t="inlineStr">
         <is>
           <t>Cliente</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="38">
-      <c r="A7" s="42" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="43">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>C. Mano de obra, retroexcavadora y dirección técnica (por un tanto)</t>
         </is>
       </c>
-      <c r="B7" s="43" t="n">
+      <c r="B7" s="48" t="n">
         <v>36000</v>
       </c>
-      <c r="C7" s="44" t="n">
+      <c r="C7" s="49" t="n">
         <v>0.368675073799917</v>
       </c>
-      <c r="D7" s="42" t="inlineStr">
+      <c r="D7" s="47" t="inlineStr">
         <is>
           <t>Pago por etapas al contratista</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="38">
-      <c r="A8" s="45" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="43">
+      <c r="A8" s="50" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="B8" s="46" t="n">
+      <c r="B8" s="51" t="n">
         <v>94711.39</v>
       </c>
-      <c r="C8" s="44" t="n">
+      <c r="C8" s="49" t="n">
         <v>0.9699369082761869</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="38">
-      <c r="A9" s="42" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="43">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>D. Imprevistos 5% (sobre A + B)</t>
         </is>
       </c>
-      <c r="B9" s="43" t="n">
+      <c r="B9" s="48" t="n">
         <v>2935.5695</v>
       </c>
-      <c r="C9" s="44" t="n">
+      <c r="C9" s="49" t="n">
         <v>0.0300630917238135</v>
       </c>
-      <c r="D9" s="42" t="inlineStr">
+      <c r="D9" s="47" t="inlineStr">
         <is>
           <t>Variaciones de precio y de metrado hasta el EMS</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="38">
-      <c r="A10" s="45" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="43">
+      <c r="A10" s="50" t="inlineStr">
         <is>
           <t>TOTAL ETAPA 1</t>
         </is>
       </c>
-      <c r="B10" s="46" t="n">
+      <c r="B10" s="51" t="n">
         <v>97646.9595</v>
       </c>
-      <c r="C10" s="44" t="n">
+      <c r="C10" s="49" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="38">
-      <c r="A11" s="42" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="43">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>Adicional: calzaduras (solo si se necesitan, se cotizan aparte)</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="47" t="inlineStr">
         <is>
           <t>por definir</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="38">
-      <c r="A13" s="47" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="43">
+      <c r="A13" s="52" t="inlineStr">
         <is>
           <t>FORMA DE PAGO DE LA MANO DE OBRA (por etapa terminada y revisada)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="31.5" customHeight="1" s="38">
-      <c r="A14" s="41" t="inlineStr">
+    <row r="14" ht="31.5" customHeight="1" s="43">
+      <c r="A14" s="46" t="inlineStr">
         <is>
           <t>Etapa</t>
         </is>
       </c>
-      <c r="B14" s="41" t="inlineStr">
+      <c r="B14" s="46" t="inlineStr">
         <is>
           <t>Monto (S/)</t>
         </is>
       </c>
-      <c r="C14" s="41" t="inlineStr">
+      <c r="C14" s="46" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D14" s="41" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="38">
-      <c r="A15" s="42" t="inlineStr">
+      <c r="D14" s="46" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="43">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>1. Limpieza, trazo, excavación con máquina, perfilado y eliminación</t>
         </is>
       </c>
-      <c r="B15" s="43" t="n">
+      <c r="B15" s="48" t="n">
         <v>5400</v>
       </c>
-      <c r="C15" s="48" t="n">
+      <c r="C15" s="53" t="n">
         <v>0.15</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="38">
-      <c r="A16" s="42" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="43">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>2. Solados, acero, encofrado y vaciado de zapatas, VE y VC</t>
         </is>
       </c>
-      <c r="B16" s="43" t="n">
+      <c r="B16" s="48" t="n">
         <v>10800</v>
       </c>
-      <c r="C16" s="48" t="n">
+      <c r="C16" s="53" t="n">
         <v>0.3</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="38">
-      <c r="A17" s="42" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="43">
+      <c r="A17" s="47" t="inlineStr">
         <is>
           <t>3. Relleno compactado y sobrecimientos</t>
         </is>
       </c>
-      <c r="B17" s="43" t="n">
+      <c r="B17" s="48" t="n">
         <v>4320</v>
       </c>
-      <c r="C17" s="48" t="n">
+      <c r="C17" s="53" t="n">
         <v>0.12</v>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="38">
-      <c r="A18" s="42" t="inlineStr">
+    <row r="18" ht="15" customHeight="1" s="43">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>4. Columnas del 1er piso hasta +2.30</t>
         </is>
       </c>
-      <c r="B18" s="43" t="n">
+      <c r="B18" s="48" t="n">
         <v>8280</v>
       </c>
-      <c r="C18" s="48" t="n">
+      <c r="C18" s="53" t="n">
         <v>0.23</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="38">
-      <c r="A19" s="42" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="43">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>5. Cerco delantero, muros del perímetro, juntas y limpieza final</t>
         </is>
       </c>
-      <c r="B19" s="43" t="n">
+      <c r="B19" s="48" t="n">
         <v>7200</v>
       </c>
-      <c r="C19" s="48" t="n">
+      <c r="C19" s="53" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="38">
-      <c r="A20" s="45" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="43">
+      <c r="A20" s="50" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B20" s="46" t="n">
+      <c r="B20" s="51" t="n">
         <v>36000</v>
       </c>
-      <c r="C20" s="49" t="n">
+      <c r="C20" s="54" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="38">
-      <c r="A22" s="50" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="43">
+      <c r="A22" s="55" t="inlineStr">
         <is>
           <t>INCLUYE: todo lo del cuadro E-10 con metrados verificados (hoja Metrados).</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="38">
-      <c r="A23" s="50" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="43">
+      <c r="A23" s="55" t="inlineStr">
         <is>
           <t>NO INCLUYE: vigas y techo del 1er piso, nudos sobre +2.30, tabiques interiores, escalera, falso piso, tarrajeos, instalaciones, fachada existente, licencia, EMS, calzaduras.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="38">
-      <c r="A24" s="50" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="43">
+      <c r="A24" s="55" t="inlineStr">
         <is>
           <t>Materiales a precio de tienda con IGV; el premezclado y la bomba deben confirmarse con 2-3 concreteras. Validez: 15 días.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="38">
-      <c r="A25" s="50" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="43">
+      <c r="A25" s="55" t="inlineStr">
         <is>
           <t>VE de -1.50 a -0.80 conectadas a las zapatas. Sistema mixto: linderos A y C de albañilería confinada (muro endentado de KK portante antes del vaciado de columnas).</t>
         </is>
@@ -941,1053 +956,1053 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="7" customWidth="1" style="37" min="1" max="1"/>
-    <col width="48" customWidth="1" style="37" min="2" max="2"/>
-    <col width="6" customWidth="1" style="37" min="3" max="3"/>
-    <col width="11" customWidth="1" style="37" min="4" max="5"/>
-    <col width="10" customWidth="1" style="37" min="6" max="6"/>
-    <col width="80" customWidth="1" style="37" min="7" max="7"/>
+    <col width="7" customWidth="1" style="42" min="1" max="1"/>
+    <col width="48" customWidth="1" style="42" min="2" max="2"/>
+    <col width="6" customWidth="1" style="42" min="3" max="3"/>
+    <col width="11" customWidth="1" style="42" min="4" max="5"/>
+    <col width="10" customWidth="1" style="42" min="6" max="6"/>
+    <col width="80" customWidth="1" style="42" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="38">
-      <c r="A1" s="39" t="inlineStr">
+    <row r="1" ht="16.15" customHeight="1" s="43">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>ETAPA 1 - METRADOS VERIFICADOS (E-10 vs. revisión)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="38">
-      <c r="A2" s="40" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="43">
+      <c r="A2" s="45" t="inlineStr">
         <is>
           <t>Revisión del cuadro E-10 contra E-01, E-02/E-03, E-04. Filas en naranja = corregidas. VE de -1.50 a -0.80 conectadas a las zapatas (tecnopor debajo entre zapatas). Sistema mixto: albañilería confinada en linderos A y C.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" s="38">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="4" ht="31.5" customHeight="1" s="43">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Ítem</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>Partida</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>Und</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Metrado E-10</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>Metrado verificado</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>Diferencia</t>
         </is>
       </c>
-      <c r="G4" s="41" t="inlineStr">
+      <c r="G4" s="46" t="inlineStr">
         <is>
           <t>Sustento de la verificación</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="38">
-      <c r="A5" s="51" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="43">
+      <c r="A5" s="56" t="inlineStr">
         <is>
           <t>01  OBRAS PRELIMINARES</t>
         </is>
       </c>
-      <c r="B5" s="52" t="n"/>
-      <c r="C5" s="52" t="n"/>
-      <c r="D5" s="52" t="n"/>
-      <c r="E5" s="52" t="n"/>
-      <c r="F5" s="52" t="n"/>
-      <c r="G5" s="52" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="38">
-      <c r="A6" s="42" t="inlineStr">
+      <c r="B5" s="57" t="n"/>
+      <c r="C5" s="57" t="n"/>
+      <c r="D5" s="57" t="n"/>
+      <c r="E5" s="57" t="n"/>
+      <c r="F5" s="57" t="n"/>
+      <c r="G5" s="57" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="43">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>01.01</t>
         </is>
       </c>
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>Limpieza de terreno</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D6" s="43" t="n">
+      <c r="D6" s="48" t="n">
         <v>170</v>
       </c>
-      <c r="E6" s="53" t="n">
+      <c r="E6" s="58" t="n">
         <v>170</v>
       </c>
-      <c r="F6" s="54" t="n">
+      <c r="F6" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="55" t="inlineStr">
+      <c r="G6" s="60" t="inlineStr">
         <is>
           <t>Lote 7.90 × 21.55</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="38">
-      <c r="A7" s="42" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="43">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>01.02</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>Trazo, nivelación y replanteo</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D7" s="43" t="n">
+      <c r="D7" s="48" t="n">
         <v>170</v>
       </c>
-      <c r="E7" s="53" t="n">
+      <c r="E7" s="58" t="n">
         <v>170</v>
       </c>
-      <c r="F7" s="54" t="n">
+      <c r="F7" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="55" t="inlineStr">
+      <c r="G7" s="60" t="inlineStr">
         <is>
           <t>Lote 7.90 × 21.55</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="38">
-      <c r="A8" s="51" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="43">
+      <c r="A8" s="56" t="inlineStr">
         <is>
           <t>02  MOVIMIENTO DE TIERRAS</t>
         </is>
       </c>
-      <c r="B8" s="52" t="n"/>
-      <c r="C8" s="52" t="n"/>
-      <c r="D8" s="52" t="n"/>
-      <c r="E8" s="52" t="n"/>
-      <c r="F8" s="52" t="n"/>
-      <c r="G8" s="52" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="38">
-      <c r="A9" s="42" t="inlineStr">
+      <c r="B8" s="57" t="n"/>
+      <c r="C8" s="57" t="n"/>
+      <c r="D8" s="57" t="n"/>
+      <c r="E8" s="57" t="n"/>
+      <c r="F8" s="57" t="n"/>
+      <c r="G8" s="57" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="43">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>02.01</t>
         </is>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="47" t="inlineStr">
         <is>
           <t>Excavación zapatas vivienda (retroexcavadora)</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D9" s="43" t="n">
+      <c r="D9" s="48" t="n">
         <v>87.09999999999999</v>
       </c>
-      <c r="E9" s="53" t="n">
+      <c r="E9" s="58" t="n">
         <v>87.09999999999999</v>
       </c>
-      <c r="F9" s="54" t="n">
+      <c r="F9" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="55" t="inlineStr">
+      <c r="G9" s="60" t="inlineStr">
         <is>
           <t>15 zapatas + 0.10 de sobreancho × 1.60 (fondo -1.50 + solado)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="22.35" customHeight="1" s="38">
-      <c r="A10" s="56" t="inlineStr">
+    <row r="10" ht="22.35" customHeight="1" s="43">
+      <c r="A10" s="61" t="inlineStr">
         <is>
           <t>02.02</t>
         </is>
       </c>
-      <c r="B10" s="56" t="inlineStr">
+      <c r="B10" s="61" t="inlineStr">
         <is>
           <t>Excavación zanjas VE / VC (retroexcavadora)</t>
         </is>
       </c>
-      <c r="C10" s="56" t="inlineStr">
+      <c r="C10" s="61" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D10" s="57" t="n">
+      <c r="D10" s="62" t="n">
         <v>24.3</v>
       </c>
-      <c r="E10" s="58" t="n">
+      <c r="E10" s="63" t="n">
         <v>32.9</v>
       </c>
-      <c r="F10" s="59" t="n">
+      <c r="F10" s="64" t="n">
         <v>8.6</v>
       </c>
-      <c r="G10" s="60" t="inlineStr">
+      <c r="G10" s="65" t="inlineStr">
         <is>
           <t>VE ahora con fondo -1.50 + tecnopor: 0.70×1.60×24.53 = 27.5; VC 0.55×1.50×6.56 = 5.4. (El modelo, descontando el sobreancho de pozos, da 28.3)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="38">
-      <c r="A11" s="56" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="43">
+      <c r="A11" s="61" t="inlineStr">
         <is>
           <t>02.03</t>
         </is>
       </c>
-      <c r="B11" s="56" t="inlineStr">
+      <c r="B11" s="61" t="inlineStr">
         <is>
           <t>Excavación manual cerco (ZC, cimiento corrido, VA)</t>
         </is>
       </c>
-      <c r="C11" s="56" t="inlineStr">
+      <c r="C11" s="61" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D11" s="57" t="n">
+      <c r="D11" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="E11" s="58" t="n">
+      <c r="E11" s="63" t="n">
         <v>13.3</v>
       </c>
-      <c r="F11" s="59" t="n">
+      <c r="F11" s="64" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="G11" s="60" t="inlineStr">
+      <c r="G11" s="65" t="inlineStr">
         <is>
           <t>E-10 omite la VA del cerco. ZC 5.04 + cimiento 2.97 + VA 5.31 (de tu Excel, E-09)</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="22.35" customHeight="1" s="38">
-      <c r="A12" s="56" t="inlineStr">
+    <row r="12" ht="22.35" customHeight="1" s="43">
+      <c r="A12" s="61" t="inlineStr">
         <is>
           <t>02.04</t>
         </is>
       </c>
-      <c r="B12" s="56" t="inlineStr">
+      <c r="B12" s="61" t="inlineStr">
         <is>
           <t>Relleno compactado con material propio hasta -0.20</t>
         </is>
       </c>
-      <c r="C12" s="56" t="inlineStr">
+      <c r="C12" s="61" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D12" s="57" t="n">
+      <c r="D12" s="62" t="n">
         <v>79.40000000000001</v>
       </c>
-      <c r="E12" s="58" t="n">
+      <c r="E12" s="63" t="n">
         <v>70.5</v>
       </c>
-      <c r="F12" s="59" t="n">
+      <c r="F12" s="64" t="n">
         <v>-8.900000000000009</v>
       </c>
-      <c r="G12" s="60" t="inlineStr">
+      <c r="G12" s="65" t="inlineStr">
         <is>
           <t>Vivienda: excavación bajo -0.20 = 104.9 - enterrado 41.7 (solado, zapatas, VE, VC, tecnopor, columnas, sobrecimiento) = 63.2; cerco 7.3</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="38">
-      <c r="A13" s="56" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="43">
+      <c r="A13" s="61" t="inlineStr">
         <is>
           <t>02.05</t>
         </is>
       </c>
-      <c r="B13" s="56" t="inlineStr">
+      <c r="B13" s="61" t="inlineStr">
         <is>
           <t>Eliminación de material excedente (esponj. 25%)</t>
         </is>
       </c>
-      <c r="C13" s="56" t="inlineStr">
+      <c r="C13" s="61" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D13" s="57" t="n">
+      <c r="D13" s="62" t="n">
         <v>53.5</v>
       </c>
-      <c r="E13" s="58" t="n">
+      <c r="E13" s="63" t="n">
         <v>78.5</v>
       </c>
-      <c r="F13" s="59" t="n">
+      <c r="F13" s="64" t="n">
         <v>25</v>
       </c>
-      <c r="G13" s="60" t="inlineStr">
+      <c r="G13" s="65" t="inlineStr">
         <is>
           <t>(133.3 - 70.5) × 1.25</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="38">
-      <c r="A14" s="51" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="43">
+      <c r="A14" s="56" t="inlineStr">
         <is>
           <t>03  CONCRETO SIMPLE</t>
         </is>
       </c>
-      <c r="B14" s="52" t="n"/>
-      <c r="C14" s="52" t="n"/>
-      <c r="D14" s="52" t="n"/>
-      <c r="E14" s="52" t="n"/>
-      <c r="F14" s="52" t="n"/>
-      <c r="G14" s="52" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="38">
-      <c r="A15" s="42" t="inlineStr">
+      <c r="B14" s="57" t="n"/>
+      <c r="C14" s="57" t="n"/>
+      <c r="D14" s="57" t="n"/>
+      <c r="E14" s="57" t="n"/>
+      <c r="F14" s="57" t="n"/>
+      <c r="G14" s="57" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="43">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>03.01</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="47" t="inlineStr">
         <is>
           <t>Solado C:H 1:12 (0.10 vivienda / 0.05 cerco)</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D15" s="43" t="n">
+      <c r="D15" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="E15" s="53" t="n">
+      <c r="E15" s="58" t="n">
         <v>50</v>
       </c>
-      <c r="F15" s="54" t="n">
+      <c r="F15" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="55" t="inlineStr">
+      <c r="G15" s="60" t="inlineStr">
         <is>
           <t>46.79 + 3.20</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="38">
-      <c r="A16" s="42" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="43">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>03.02</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="47" t="inlineStr">
         <is>
           <t>Cimiento corrido ciclópeo 1:10 + 30% PG (cerco)</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D16" s="43" t="n">
+      <c r="D16" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="E16" s="53" t="n">
+      <c r="E16" s="58" t="n">
         <v>2.2</v>
       </c>
-      <c r="F16" s="54" t="n">
+      <c r="F16" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="55" t="inlineStr">
+      <c r="G16" s="60" t="inlineStr">
         <is>
           <t>9.28 × 0.40 × 0.60</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22.35" customHeight="1" s="38">
-      <c r="A17" s="56" t="inlineStr">
+    <row r="17" ht="22.35" customHeight="1" s="43">
+      <c r="A17" s="61" t="inlineStr">
         <is>
           <t>03.03</t>
         </is>
       </c>
-      <c r="B17" s="56" t="inlineStr">
+      <c r="B17" s="61" t="inlineStr">
         <is>
           <t>Sobrecimiento 1:8 + 25% PM 0.15 de ancho (perímetro + cerco)</t>
         </is>
       </c>
-      <c r="C17" s="56" t="inlineStr">
+      <c r="C17" s="61" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D17" s="57" t="n">
+      <c r="D17" s="62" t="n">
         <v>2.7</v>
       </c>
-      <c r="E17" s="58" t="n">
+      <c r="E17" s="63" t="n">
         <v>5.85</v>
       </c>
-      <c r="F17" s="59" t="n">
+      <c r="F17" s="64" t="n">
         <v>3.15</v>
       </c>
-      <c r="G17" s="60" t="inlineStr">
+      <c r="G17" s="65" t="inlineStr">
         <is>
           <t>Arranca desde la viga: sobre VE (top -0.80) h = 1.00 → 20.98 m; sobre VC de ejes A y C (top -1.10 / zapata -1.00) h 1.20-1.30 → 10.72 m; cerco h = 0.40 → 11.78 m (medido en el modelo)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="38">
-      <c r="A18" s="56" t="inlineStr">
+    <row r="18" ht="15" customHeight="1" s="43">
+      <c r="A18" s="61" t="inlineStr">
         <is>
           <t>03.04</t>
         </is>
       </c>
-      <c r="B18" s="56" t="inlineStr">
+      <c r="B18" s="61" t="inlineStr">
         <is>
           <t>Encofrado de sobrecimiento (2 caras)</t>
         </is>
       </c>
-      <c r="C18" s="56" t="inlineStr">
+      <c r="C18" s="61" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D18" s="57" t="n">
+      <c r="D18" s="62" t="n">
         <v>35.4</v>
       </c>
-      <c r="E18" s="58" t="n">
+      <c r="E18" s="63" t="n">
         <v>78</v>
       </c>
-      <c r="F18" s="59" t="n">
+      <c r="F18" s="64" t="n">
         <v>42.6</v>
       </c>
-      <c r="G18" s="60" t="inlineStr">
+      <c r="G18" s="65" t="inlineStr">
         <is>
           <t>2 × (1.00 × 20.98 + 1.25 × 10.72 + 0.40 × 11.78)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="38">
-      <c r="A19" s="51" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="43">
+      <c r="A19" s="56" t="inlineStr">
         <is>
           <t>04  CONCRETO ARMADO f'c 210</t>
         </is>
       </c>
-      <c r="B19" s="52" t="n"/>
-      <c r="C19" s="52" t="n"/>
-      <c r="D19" s="52" t="n"/>
-      <c r="E19" s="52" t="n"/>
-      <c r="F19" s="52" t="n"/>
-      <c r="G19" s="52" t="n"/>
-    </row>
-    <row r="20" ht="22.35" customHeight="1" s="38">
-      <c r="A20" s="42" t="inlineStr">
+      <c r="B19" s="57" t="n"/>
+      <c r="C19" s="57" t="n"/>
+      <c r="D19" s="57" t="n"/>
+      <c r="E19" s="57" t="n"/>
+      <c r="F19" s="57" t="n"/>
+      <c r="G19" s="57" t="n"/>
+    </row>
+    <row r="20" ht="22.35" customHeight="1" s="43">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>04.01</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Zapatas Z-1 a Z-5 (vaciado contra terreno)</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D20" s="43" t="n">
+      <c r="D20" s="48" t="n">
         <v>23.4</v>
       </c>
-      <c r="E20" s="53" t="n">
+      <c r="E20" s="58" t="n">
         <v>23.4</v>
       </c>
-      <c r="F20" s="54" t="n">
+      <c r="F20" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="55" t="inlineStr">
+      <c r="G20" s="60" t="inlineStr">
         <is>
           <t>Cuadro E-01. OJO: la excavación lleva 0.10 de sobreancho; si se vacía contra terreno, ese hueco se llena de concreto (+3.8 m³). Perfilar a la medida exacta los 0.50 inferiores</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="22.35" customHeight="1" s="38">
-      <c r="A21" s="56" t="inlineStr">
+    <row r="21" ht="22.35" customHeight="1" s="43">
+      <c r="A21" s="61" t="inlineStr">
         <is>
           <t>04.02</t>
         </is>
       </c>
-      <c r="B21" s="56" t="inlineStr">
+      <c r="B21" s="61" t="inlineStr">
         <is>
           <t>Vigas de equilibrio VE 0.30×0.70 (de -1.50 a -0.80)</t>
         </is>
       </c>
-      <c r="C21" s="56" t="inlineStr">
+      <c r="C21" s="61" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D21" s="57" t="n">
+      <c r="D21" s="62" t="n">
         <v>5.2</v>
       </c>
-      <c r="E21" s="58" t="n">
+      <c r="E21" s="63" t="n">
         <v>7.01</v>
       </c>
-      <c r="F21" s="59" t="n">
+      <c r="F21" s="64" t="n">
         <v>1.81</v>
       </c>
-      <c r="G21" s="60" t="inlineStr">
+      <c r="G21" s="65" t="inlineStr">
         <is>
           <t>Entre zapatas 0.30×0.70×24.53 = 5.15 + sobre zapata solo lo que sobresale (-1.00 a -0.80) 0.30×0.20×30.95 = 1.86</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="38">
-      <c r="A22" s="56" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="43">
+      <c r="A22" s="61" t="inlineStr">
         <is>
           <t>04.03</t>
         </is>
       </c>
-      <c r="B22" s="56" t="inlineStr">
+      <c r="B22" s="61" t="inlineStr">
         <is>
           <t>Encofrado VE (2 caras)</t>
         </is>
       </c>
-      <c r="C22" s="56" t="inlineStr">
+      <c r="C22" s="61" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D22" s="57" t="n">
+      <c r="D22" s="62" t="n">
         <v>34.4</v>
       </c>
-      <c r="E22" s="58" t="n">
+      <c r="E22" s="63" t="n">
         <v>46.7</v>
       </c>
-      <c r="F22" s="59" t="n">
+      <c r="F22" s="64" t="n">
         <v>12.3</v>
       </c>
-      <c r="G22" s="60" t="inlineStr">
+      <c r="G22" s="65" t="inlineStr">
         <is>
           <t>2 × 0.70 × 24.53 + 2 × 0.20 × 30.95</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="38">
-      <c r="A23" s="42" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="43">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>04.04</t>
         </is>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B23" s="47" t="inlineStr">
         <is>
           <t>Tecnopor e = 0.10 bajo VE (solo entre zapatas, de -1.60 a -1.50)</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C23" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D23" s="43" t="n">
+      <c r="D23" s="48" t="n">
         <v>7.4</v>
       </c>
-      <c r="E23" s="53" t="n">
+      <c r="E23" s="58" t="n">
         <v>7.4</v>
       </c>
-      <c r="F23" s="54" t="n">
+      <c r="F23" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="55" t="inlineStr">
+      <c r="G23" s="60" t="inlineStr">
         <is>
           <t>0.30 × 24.53</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="38">
-      <c r="A24" s="42" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="43">
+      <c r="A24" s="47" t="inlineStr">
         <is>
           <t>04.05</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B24" s="47" t="inlineStr">
         <is>
           <t>Vigas de conexión VC 0.25×0.40</t>
         </is>
       </c>
-      <c r="C24" s="42" t="inlineStr">
+      <c r="C24" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D24" s="43" t="n">
+      <c r="D24" s="48" t="n">
         <v>0.7</v>
       </c>
-      <c r="E24" s="53" t="n">
+      <c r="E24" s="58" t="n">
         <v>0.66</v>
       </c>
-      <c r="F24" s="54" t="n">
+      <c r="F24" s="59" t="n">
         <v>-0.0399999999999999</v>
       </c>
-      <c r="G24" s="55" t="inlineStr">
+      <c r="G24" s="60" t="inlineStr">
         <is>
           <t>0.10 × 6.56 (sobre zapata queda dentro de la zapata)</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="38">
-      <c r="A25" s="42" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="43">
+      <c r="A25" s="47" t="inlineStr">
         <is>
           <t>04.05b</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B25" s="47" t="inlineStr">
         <is>
           <t>Encofrado VC</t>
         </is>
       </c>
-      <c r="C25" s="42" t="inlineStr">
+      <c r="C25" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D25" s="43" t="n">
+      <c r="D25" s="48" t="n">
         <v>5.2</v>
       </c>
-      <c r="E25" s="53" t="n">
+      <c r="E25" s="58" t="n">
         <v>5.2</v>
       </c>
-      <c r="F25" s="54" t="n">
+      <c r="F25" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="55" t="inlineStr">
+      <c r="G25" s="60" t="inlineStr">
         <is>
           <t>2 × 0.40 × 6.56</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="38">
-      <c r="A26" s="42" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="43">
+      <c r="A26" s="47" t="inlineStr">
         <is>
           <t>04.06</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B26" s="47" t="inlineStr">
         <is>
           <t>Columnas 1er piso (-1.00 a +2.30)</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C26" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D26" s="43" t="n">
+      <c r="D26" s="48" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E26" s="53" t="n">
+      <c r="E26" s="58" t="n">
         <v>8.32</v>
       </c>
-      <c r="F26" s="54" t="n">
+      <c r="F26" s="59" t="n">
         <v>0.120000000000001</v>
       </c>
-      <c r="G26" s="55" t="inlineStr">
+      <c r="G26" s="60" t="inlineStr">
         <is>
           <t>2.49 m² × 3.30 = 8.22 + 0.10 de concreto que entra en los dientes del muro</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="38">
-      <c r="A27" s="56" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="43">
+      <c r="A27" s="61" t="inlineStr">
         <is>
           <t>04.07</t>
         </is>
       </c>
-      <c r="B27" s="56" t="inlineStr">
+      <c r="B27" s="61" t="inlineStr">
         <is>
           <t>Encofrado columnas 1er piso</t>
         </is>
       </c>
-      <c r="C27" s="56" t="inlineStr">
+      <c r="C27" s="61" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D27" s="57" t="n">
+      <c r="D27" s="62" t="n">
         <v>83.5</v>
       </c>
-      <c r="E27" s="58" t="n">
+      <c r="E27" s="63" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="F27" s="59" t="n">
+      <c r="F27" s="64" t="n">
         <v>-4.40000000000001</v>
       </c>
-      <c r="G27" s="60" t="inlineStr">
+      <c r="G27" s="65" t="inlineStr">
         <is>
           <t>25.3 m × 3.30 = 83.5 - 16 caras contra muro endentado (0.13 × 2.10) = 4.4</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="38">
-      <c r="A28" s="42" t="inlineStr">
+    <row r="28" ht="15" customHeight="1" s="43">
+      <c r="A28" s="47" t="inlineStr">
         <is>
           <t>04.08</t>
         </is>
       </c>
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B28" s="47" t="inlineStr">
         <is>
           <t>Cerco: ZC, VA, CA, solera</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C28" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D28" s="43" t="n">
+      <c r="D28" s="48" t="n">
         <v>3.5</v>
       </c>
-      <c r="E28" s="53" t="n">
+      <c r="E28" s="58" t="n">
         <v>3.5</v>
       </c>
-      <c r="F28" s="54" t="n">
+      <c r="F28" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="55" t="inlineStr">
+      <c r="G28" s="60" t="inlineStr">
         <is>
           <t>E-09 (no verificado: plano no recibido)</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="38">
-      <c r="A29" s="42" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="43">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>04.08b</t>
         </is>
       </c>
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>Encofrado cerco</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D29" s="43" t="n">
+      <c r="D29" s="48" t="n">
         <v>21.9</v>
       </c>
-      <c r="E29" s="53" t="n">
+      <c r="E29" s="58" t="n">
         <v>21.9</v>
       </c>
-      <c r="F29" s="54" t="n">
+      <c r="F29" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="55" t="inlineStr">
+      <c r="G29" s="60" t="inlineStr">
         <is>
           <t>E-09 (no verificado)</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="22.35" customHeight="1" s="38">
-      <c r="A30" s="56" t="inlineStr">
+    <row r="30" ht="22.35" customHeight="1" s="43">
+      <c r="A30" s="61" t="inlineStr">
         <is>
           <t>04.09</t>
         </is>
       </c>
-      <c r="B30" s="56" t="inlineStr">
+      <c r="B30" s="61" t="inlineStr">
         <is>
           <t>Acero fy 4200 habilitado y colocado</t>
         </is>
       </c>
-      <c r="C30" s="56" t="inlineStr">
+      <c r="C30" s="61" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D30" s="57" t="n">
+      <c r="D30" s="62" t="n">
         <v>4881</v>
       </c>
-      <c r="E30" s="58" t="n">
+      <c r="E30" s="63" t="n">
         <v>5870</v>
       </c>
-      <c r="F30" s="59" t="n">
+      <c r="F30" s="64" t="n">
         <v>989</v>
       </c>
-      <c r="G30" s="60" t="inlineStr">
+      <c r="G30" s="65" t="inlineStr">
         <is>
           <t>E-10 pone VE 956 y VC 153 kg. Cuadro de vigas E-02/E-03: VE 1,815 y VC 282 kg (barras continuas con ganchos de 0.45 en columnas)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="38">
-      <c r="A31" s="42" t="inlineStr">
+    <row r="31" ht="15" customHeight="1" s="43">
+      <c r="A31" s="47" t="inlineStr">
         <is>
           <t>04.10</t>
         </is>
       </c>
-      <c r="B31" s="42" t="inlineStr">
+      <c r="B31" s="47" t="inlineStr">
         <is>
           <t>Anclaje con epóxico Ø3/8" en columnas existentes</t>
         </is>
       </c>
-      <c r="C31" s="42" t="inlineStr">
+      <c r="C31" s="47" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D31" s="43" t="n">
+      <c r="D31" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="E31" s="53" t="n">
+      <c r="E31" s="58" t="n">
         <v>8</v>
       </c>
-      <c r="F31" s="54" t="n">
+      <c r="F31" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="55" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="38">
-      <c r="A32" s="51" t="inlineStr">
+      <c r="G31" s="60" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="43">
+      <c r="A32" s="56" t="inlineStr">
         <is>
           <t>05  ALBAÑILERÍA KK 18 huecos de soga, mortero 1:4</t>
         </is>
       </c>
-      <c r="B32" s="52" t="n"/>
-      <c r="C32" s="52" t="n"/>
-      <c r="D32" s="52" t="n"/>
-      <c r="E32" s="52" t="n"/>
-      <c r="F32" s="52" t="n"/>
-      <c r="G32" s="52" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="38">
-      <c r="A33" s="42" t="inlineStr">
+      <c r="B32" s="57" t="n"/>
+      <c r="C32" s="57" t="n"/>
+      <c r="D32" s="57" t="n"/>
+      <c r="E32" s="57" t="n"/>
+      <c r="F32" s="57" t="n"/>
+      <c r="G32" s="57" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="43">
+      <c r="A33" s="47" t="inlineStr">
         <is>
           <t>05.01</t>
         </is>
       </c>
-      <c r="B33" s="42" t="inlineStr">
+      <c r="B33" s="47" t="inlineStr">
         <is>
           <t>Muro cerco delantero</t>
         </is>
       </c>
-      <c r="C33" s="42" t="inlineStr">
+      <c r="C33" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D33" s="43" t="n">
+      <c r="D33" s="48" t="n">
         <v>29.8</v>
       </c>
-      <c r="E33" s="53" t="n">
+      <c r="E33" s="58" t="n">
         <v>29.8</v>
       </c>
-      <c r="F33" s="54" t="n">
+      <c r="F33" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G33" s="55" t="inlineStr">
+      <c r="G33" s="60" t="inlineStr">
         <is>
           <t>E-09 (no verificado)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="38">
-      <c r="A34" s="56" t="inlineStr">
+    <row r="34" ht="15" customHeight="1" s="43">
+      <c r="A34" s="61" t="inlineStr">
         <is>
           <t>05.02a</t>
         </is>
       </c>
-      <c r="B34" s="56" t="inlineStr">
+      <c r="B34" s="61" t="inlineStr">
         <is>
           <t>Muro portante linderos A y C - KK PORTANTE endentado (albañilería confinada)</t>
         </is>
       </c>
-      <c r="C34" s="56" t="inlineStr">
+      <c r="C34" s="61" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D34" s="57" t="n">
+      <c r="D34" s="62" t="n">
         <v>57.1</v>
       </c>
-      <c r="E34" s="58" t="n">
+      <c r="E34" s="63" t="n">
         <v>52.5</v>
       </c>
-      <c r="F34" s="59" t="n">
+      <c r="F34" s="64" t="n">
         <v>-4.6</v>
       </c>
-      <c r="G34" s="60" t="inlineStr">
+      <c r="G34" s="65" t="inlineStr">
         <is>
           <t>2 × 12.50 × 2.10 (de +0.20 a +2.30). Se levanta ANTES de vaciar las columnas</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="38">
-      <c r="A35" s="56" t="inlineStr">
+    <row r="35" ht="15" customHeight="1" s="43">
+      <c r="A35" s="61" t="inlineStr">
         <is>
           <t>05.02b</t>
         </is>
       </c>
-      <c r="B35" s="56" t="inlineStr">
+      <c r="B35" s="61" t="inlineStr">
         <is>
           <t>Muro fondo eje 5 - tabique KK 18 huecos con junta</t>
         </is>
       </c>
-      <c r="C35" s="56" t="inlineStr">
+      <c r="C35" s="61" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D35" s="57" t="n">
+      <c r="D35" s="62" t="n">
         <v>0</v>
       </c>
-      <c r="E35" s="58" t="n">
+      <c r="E35" s="63" t="n">
         <v>14.1</v>
       </c>
-      <c r="F35" s="59" t="n">
+      <c r="F35" s="64" t="n">
         <v>14.1</v>
       </c>
-      <c r="G35" s="60" t="inlineStr">
+      <c r="G35" s="65" t="inlineStr">
         <is>
           <t>6.70 × 2.10</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="38">
-      <c r="A36" s="56" t="inlineStr">
+    <row r="36" ht="15" customHeight="1" s="43">
+      <c r="A36" s="61" t="inlineStr">
         <is>
           <t>05.03</t>
         </is>
       </c>
-      <c r="B36" s="56" t="inlineStr">
+      <c r="B36" s="61" t="inlineStr">
         <is>
           <t>Junta con tecnopor 1" (solo fondo y encuentro cerco-vivienda)</t>
         </is>
       </c>
-      <c r="C36" s="56" t="inlineStr">
+      <c r="C36" s="61" t="inlineStr">
         <is>
           <t>ml</t>
         </is>
       </c>
-      <c r="D36" s="57" t="n">
+      <c r="D36" s="62" t="n">
         <v>42</v>
       </c>
-      <c r="E36" s="58" t="n">
+      <c r="E36" s="63" t="n">
         <v>13.6</v>
       </c>
-      <c r="F36" s="59" t="n">
+      <c r="F36" s="64" t="n">
         <v>-28.4</v>
       </c>
-      <c r="G36" s="60" t="inlineStr">
+      <c r="G36" s="65" t="inlineStr">
         <is>
           <t>Linderos ya no llevan junta (muro endentado). Fondo 4 × 2.10 + cerco-vivienda 2 × 2.60</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="38">
-      <c r="A37" s="51" t="inlineStr">
+    <row r="37" ht="15" customHeight="1" s="43">
+      <c r="A37" s="56" t="inlineStr">
         <is>
           <t>06  VARIOS</t>
         </is>
       </c>
-      <c r="B37" s="52" t="n"/>
-      <c r="C37" s="52" t="n"/>
-      <c r="D37" s="52" t="n"/>
-      <c r="E37" s="52" t="n"/>
-      <c r="F37" s="52" t="n"/>
-      <c r="G37" s="52" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="38">
-      <c r="A38" s="42" t="inlineStr">
+      <c r="B37" s="57" t="n"/>
+      <c r="C37" s="57" t="n"/>
+      <c r="D37" s="57" t="n"/>
+      <c r="E37" s="57" t="n"/>
+      <c r="F37" s="57" t="n"/>
+      <c r="G37" s="57" t="n"/>
+    </row>
+    <row r="38" ht="15" customHeight="1" s="43">
+      <c r="A38" s="47" t="inlineStr">
         <is>
           <t>06.01</t>
         </is>
       </c>
-      <c r="B38" s="42" t="inlineStr">
+      <c r="B38" s="47" t="inlineStr">
         <is>
           <t>Curado de concreto</t>
         </is>
       </c>
-      <c r="C38" s="42" t="inlineStr">
+      <c r="C38" s="47" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D38" s="43" t="n">
+      <c r="D38" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="E38" s="53" t="n">
+      <c r="E38" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="F38" s="54" t="n">
+      <c r="F38" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="55" t="n"/>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="38">
-      <c r="A39" s="42" t="inlineStr">
+      <c r="G38" s="60" t="n"/>
+    </row>
+    <row r="39" ht="15" customHeight="1" s="43">
+      <c r="A39" s="47" t="inlineStr">
         <is>
           <t>06.02</t>
         </is>
       </c>
-      <c r="B39" s="42" t="inlineStr">
+      <c r="B39" s="47" t="inlineStr">
         <is>
           <t>Ensayo de probetas</t>
         </is>
       </c>
-      <c r="C39" s="42" t="inlineStr">
+      <c r="C39" s="47" t="inlineStr">
         <is>
           <t>juego</t>
         </is>
       </c>
-      <c r="D39" s="43" t="n">
+      <c r="D39" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="E39" s="53" t="n">
+      <c r="E39" s="58" t="n">
         <v>5</v>
       </c>
-      <c r="F39" s="54" t="n">
+      <c r="F39" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="G39" s="55" t="n"/>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="38">
-      <c r="A41" s="61" t="inlineStr">
+      <c r="G39" s="60" t="n"/>
+    </row>
+    <row r="41" ht="15" customHeight="1" s="43">
+      <c r="A41" s="66" t="inlineStr">
         <is>
           <t>CAMBIOS DE OBRA: VE de -1.50 a -0.80 conectadas a las zapatas (tecnopor 0.10 bajo VE entre zapatas, excavación a -1.60).</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="15" customHeight="1" s="38">
-      <c r="A42" s="61" t="inlineStr">
+    <row r="42" ht="15" customHeight="1" s="43">
+      <c r="A42" s="66" t="inlineStr">
         <is>
           <t>Sistema mixto: linderos A y C de albañilería confinada (KK portante con ≤30% vacíos, E.070), muro endentado y luego vaciado de columnas.</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="15" customHeight="1" s="38">
-      <c r="A43" s="61" t="inlineStr">
+    <row r="43" ht="15" customHeight="1" s="43">
+      <c r="A43" s="66" t="inlineStr">
         <is>
           <t>Acero de columnas 1er piso: 2,646 kg (E-10) verificado (barras Ø5/8" de 6.00 m de arranque + estribos Ø1/2" 1,342 kg + montaje 3/8" 38 kg).</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="15" customHeight="1" s="38">
-      <c r="A44" s="61" t="inlineStr">
+    <row r="44" ht="15" customHeight="1" s="43">
+      <c r="A44" s="66" t="inlineStr">
         <is>
           <t>Diferencias menores a favor (no se cambian): zanjas de VE medidas sin descontar el sobreancho de los pozos (~2.5 m³ de más); encofrado de columnas sin descontar las caras donde llega la VE (~6.7 m²).</t>
         </is>
@@ -2009,800 +2024,800 @@
   <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="5" customWidth="1" style="37" min="1" max="1"/>
-    <col width="58" customWidth="1" style="37" min="2" max="2"/>
-    <col width="8" customWidth="1" style="37" min="3" max="3"/>
-    <col width="10" customWidth="1" style="37" min="4" max="5"/>
-    <col width="12" customWidth="1" style="37" min="6" max="6"/>
-    <col width="70" customWidth="1" style="37" min="7" max="7"/>
+    <col width="5" customWidth="1" style="42" min="1" max="1"/>
+    <col width="58" customWidth="1" style="42" min="2" max="2"/>
+    <col width="8" customWidth="1" style="42" min="3" max="3"/>
+    <col width="10" customWidth="1" style="42" min="4" max="5"/>
+    <col width="12" customWidth="1" style="42" min="6" max="6"/>
+    <col width="70" customWidth="1" style="42" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="38">
-      <c r="A1" s="39" t="inlineStr">
+    <row r="1" ht="16.15" customHeight="1" s="43">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>MATERIALES - ETAPA 1 (cantidades por despiece real de varillas)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="38">
-      <c r="A2" s="40" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="43">
+      <c r="A2" s="45" t="inlineStr">
         <is>
           <t>Concreto estructural con premezclado + bomba. Mezclas menores (solado, ciclópeo, sobrecimiento, solera, mortero) en obra.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="31.5" customHeight="1" s="38">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="4" ht="31.5" customHeight="1" s="43">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>Und</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>P.U. (S/)</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>Parcial (S/)</t>
         </is>
       </c>
-      <c r="G4" s="41" t="inlineStr">
+      <c r="G4" s="46" t="inlineStr">
         <is>
           <t>Cómo se calculó</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="38">
-      <c r="A5" s="51" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="43">
+      <c r="A5" s="56" t="inlineStr">
         <is>
           <t>A. CONCRETO PREMEZCLADO</t>
         </is>
       </c>
-      <c r="B5" s="52" t="n"/>
-      <c r="C5" s="52" t="n"/>
-      <c r="D5" s="52" t="n"/>
-      <c r="E5" s="52" t="n"/>
-      <c r="F5" s="52" t="n"/>
-      <c r="G5" s="52" t="n"/>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="38">
-      <c r="A6" s="42" t="n">
+      <c r="B5" s="57" t="n"/>
+      <c r="C5" s="57" t="n"/>
+      <c r="D5" s="57" t="n"/>
+      <c r="E5" s="57" t="n"/>
+      <c r="F5" s="57" t="n"/>
+      <c r="G5" s="57" t="n"/>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="43">
+      <c r="A6" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>Premezclado f'c 210 - vaciado 1: zapatas + VE + VC + ZC + VA cerco</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D6" s="62" t="n">
+      <c r="D6" s="67" t="n">
         <v>37</v>
       </c>
-      <c r="E6" s="43" t="n">
+      <c r="E6" s="48" t="n">
         <v>320</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="48" t="n">
         <v>11840</v>
       </c>
-      <c r="G6" s="42" t="inlineStr">
+      <c r="G6" s="47" t="inlineStr">
         <is>
           <t>(23.39 + 7.01 + 0.66 + 1.36 + 1.18) × 1.04 = 34.9 + 2.0 por sobreexcavación de la retro → 37.0</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="38">
-      <c r="A7" s="42" t="n">
+    <row r="7" ht="15" customHeight="1" s="43">
+      <c r="A7" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>Bomba - vaciado 1</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D7" s="62" t="n">
+      <c r="D7" s="67" t="n">
         <v>37</v>
       </c>
-      <c r="E7" s="43" t="n">
+      <c r="E7" s="48" t="n">
         <v>38</v>
       </c>
-      <c r="F7" s="43" t="n">
+      <c r="F7" s="48" t="n">
         <v>1406</v>
       </c>
-      <c r="G7" s="42" t="n"/>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="38">
-      <c r="A8" s="42" t="n">
+      <c r="G7" s="47" t="n"/>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="43">
+      <c r="A8" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Premezclado f'c 210 - vaciado 2: columnas 1er piso + CA cerco</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D8" s="62" t="n">
+      <c r="D8" s="67" t="n">
         <v>9.5</v>
       </c>
-      <c r="E8" s="43" t="n">
+      <c r="E8" s="48" t="n">
         <v>320</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="48" t="n">
         <v>3040</v>
       </c>
-      <c r="G8" s="42" t="inlineStr">
+      <c r="G8" s="47" t="inlineStr">
         <is>
           <t>(8.22 + 0.60) × 1.04 = 9.2 → pedir 9.5</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="38">
-      <c r="A9" s="42" t="n">
+    <row r="9" ht="15" customHeight="1" s="43">
+      <c r="A9" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="47" t="inlineStr">
         <is>
           <t>Bomba - vaciado 2 (cobra mínimo 20 m³)</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D9" s="62" t="n">
+      <c r="D9" s="67" t="n">
         <v>20</v>
       </c>
-      <c r="E9" s="43" t="n">
+      <c r="E9" s="48" t="n">
         <v>38</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F9" s="48" t="n">
         <v>760</v>
       </c>
-      <c r="G9" s="42" t="inlineStr">
+      <c r="G9" s="47" t="inlineStr">
         <is>
           <t>Columnas de 3.30 m: el mixer solo no llega</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="38">
-      <c r="A10" s="51" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="43">
+      <c r="A10" s="56" t="inlineStr">
         <is>
           <t>B. MEZCLAS EN OBRA</t>
         </is>
       </c>
-      <c r="B10" s="52" t="n"/>
-      <c r="C10" s="52" t="n"/>
-      <c r="D10" s="52" t="n"/>
-      <c r="E10" s="52" t="n"/>
-      <c r="F10" s="52" t="n"/>
-      <c r="G10" s="52" t="n"/>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="38">
-      <c r="A11" s="42" t="n">
+      <c r="B10" s="57" t="n"/>
+      <c r="C10" s="57" t="n"/>
+      <c r="D10" s="57" t="n"/>
+      <c r="E10" s="57" t="n"/>
+      <c r="F10" s="57" t="n"/>
+      <c r="G10" s="57" t="n"/>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="43">
+      <c r="A11" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="47" t="inlineStr">
         <is>
           <t>Cemento (solado, ciclópeo, sobrecimiento, solera, mortero)</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr">
+      <c r="C11" s="47" t="inlineStr">
         <is>
           <t>bolsa</t>
         </is>
       </c>
-      <c r="D11" s="62" t="n">
+      <c r="D11" s="67" t="n">
         <v>73</v>
       </c>
-      <c r="E11" s="43" t="n">
+      <c r="E11" s="48" t="n">
         <v>28.6</v>
       </c>
-      <c r="F11" s="43" t="n">
+      <c r="F11" s="48" t="n">
         <v>2087.8</v>
       </c>
-      <c r="G11" s="42" t="inlineStr">
+      <c r="G11" s="47" t="inlineStr">
         <is>
           <t>Solado 17 + ciclópeo 7 + sobrecim. 23 + solera 4 + mortero 22</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="38">
-      <c r="A12" s="42" t="n">
+    <row r="12" ht="15" customHeight="1" s="43">
+      <c r="A12" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="42" t="inlineStr">
+      <c r="B12" s="47" t="inlineStr">
         <is>
           <t>Hormigón (solado, ciclópeo, sobrecimiento)</t>
         </is>
       </c>
-      <c r="C12" s="42" t="inlineStr">
+      <c r="C12" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D12" s="62" t="n">
+      <c r="D12" s="67" t="n">
         <v>12.4</v>
       </c>
-      <c r="E12" s="43" t="n">
+      <c r="E12" s="48" t="n">
         <v>60</v>
       </c>
-      <c r="F12" s="43" t="n">
+      <c r="F12" s="48" t="n">
         <v>744</v>
       </c>
-      <c r="G12" s="42" t="inlineStr">
+      <c r="G12" s="47" t="inlineStr">
         <is>
           <t>5.4 + 1.9 + 5.1</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="38">
-      <c r="A13" s="42" t="n">
+    <row r="13" ht="15" customHeight="1" s="43">
+      <c r="A13" s="47" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="42" t="inlineStr">
+      <c r="B13" s="47" t="inlineStr">
         <is>
           <t>Arena gruesa (solera + mortero de muros)</t>
         </is>
       </c>
-      <c r="C13" s="42" t="inlineStr">
+      <c r="C13" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D13" s="62" t="n">
+      <c r="D13" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="43" t="n">
+      <c r="E13" s="48" t="n">
         <v>65</v>
       </c>
-      <c r="F13" s="43" t="n">
+      <c r="F13" s="48" t="n">
         <v>195</v>
       </c>
-      <c r="G13" s="42" t="inlineStr">
+      <c r="G13" s="47" t="inlineStr">
         <is>
           <t>0.2 + 96.6 m² × 0.028</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="38">
-      <c r="A14" s="42" t="n">
+    <row r="14" ht="15" customHeight="1" s="43">
+      <c r="A14" s="47" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="47" t="inlineStr">
         <is>
           <t>Piedra chancada 1/2" (solera)</t>
         </is>
       </c>
-      <c r="C14" s="42" t="inlineStr">
+      <c r="C14" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D14" s="62" t="n">
+      <c r="D14" s="67" t="n">
         <v>0.2</v>
       </c>
-      <c r="E14" s="43" t="n">
+      <c r="E14" s="48" t="n">
         <v>80</v>
       </c>
-      <c r="F14" s="43" t="n">
+      <c r="F14" s="48" t="n">
         <v>16</v>
       </c>
-      <c r="G14" s="42" t="n"/>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="38">
-      <c r="A15" s="42" t="n">
+      <c r="G14" s="47" t="n"/>
+    </row>
+    <row r="15" ht="15" customHeight="1" s="43">
+      <c r="A15" s="47" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="47" t="inlineStr">
         <is>
           <t>Piedra grande 6" (ciclópeo 30%)</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D15" s="62" t="n">
+      <c r="D15" s="67" t="n">
         <v>1.2</v>
       </c>
-      <c r="E15" s="43" t="n">
+      <c r="E15" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="F15" s="43" t="n">
+      <c r="F15" s="48" t="n">
         <v>60</v>
       </c>
-      <c r="G15" s="42" t="n"/>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="38">
-      <c r="A16" s="42" t="n">
+      <c r="G15" s="47" t="n"/>
+    </row>
+    <row r="16" ht="15" customHeight="1" s="43">
+      <c r="A16" s="47" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="47" t="inlineStr">
         <is>
           <t>Piedra mediana 4" (sobrecimiento 25%)</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D16" s="62" t="n">
+      <c r="D16" s="67" t="n">
         <v>2.3</v>
       </c>
-      <c r="E16" s="43" t="n">
+      <c r="E16" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="F16" s="43" t="n">
+      <c r="F16" s="48" t="n">
         <v>115</v>
       </c>
-      <c r="G16" s="42" t="n"/>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="38">
-      <c r="A17" s="51" t="inlineStr">
+      <c r="G16" s="47" t="n"/>
+    </row>
+    <row r="17" ht="15" customHeight="1" s="43">
+      <c r="A17" s="56" t="inlineStr">
         <is>
           <t>C. ACERO (por despiece de barras de 9 m, no por kg)</t>
         </is>
       </c>
-      <c r="B17" s="52" t="n"/>
-      <c r="C17" s="52" t="n"/>
-      <c r="D17" s="52" t="n"/>
-      <c r="E17" s="52" t="n"/>
-      <c r="F17" s="52" t="n"/>
-      <c r="G17" s="52" t="n"/>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="38">
-      <c r="A18" s="42" t="n">
+      <c r="B17" s="57" t="n"/>
+      <c r="C17" s="57" t="n"/>
+      <c r="D17" s="57" t="n"/>
+      <c r="E17" s="57" t="n"/>
+      <c r="F17" s="57" t="n"/>
+      <c r="G17" s="57" t="n"/>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="43">
+      <c r="A18" s="47" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="47" t="inlineStr">
         <is>
           <t>Varilla Ø3/4" × 9 m</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C18" s="47" t="inlineStr">
         <is>
           <t>varilla</t>
         </is>
       </c>
-      <c r="D18" s="62" t="n">
+      <c r="D18" s="67" t="n">
         <v>72</v>
       </c>
-      <c r="E18" s="43" t="n">
+      <c r="E18" s="48" t="n">
         <v>80.02</v>
       </c>
-      <c r="F18" s="43" t="n">
+      <c r="F18" s="48" t="n">
         <v>5761.44</v>
       </c>
-      <c r="G18" s="42" t="inlineStr">
+      <c r="G18" s="47" t="inlineStr">
         <is>
           <t>VE en ejes 1-5 continua (8.8 m = 1 varilla por barra): 32; VE en ejes A, B, C: 40</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="38">
-      <c r="A19" s="42" t="n">
+    <row r="19" ht="15" customHeight="1" s="43">
+      <c r="A19" s="47" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="47" t="inlineStr">
         <is>
           <t>Varilla Ø5/8" × 9 m</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="47" t="inlineStr">
         <is>
           <t>varilla</t>
         </is>
       </c>
-      <c r="D19" s="62" t="n">
+      <c r="D19" s="67" t="n">
         <v>207</v>
       </c>
-      <c r="E19" s="43" t="n">
+      <c r="E19" s="48" t="n">
         <v>54.41</v>
       </c>
-      <c r="F19" s="43" t="n">
+      <c r="F19" s="48" t="n">
         <v>11262.87</v>
       </c>
-      <c r="G19" s="42" t="inlineStr">
+      <c r="G19" s="47" t="inlineStr">
         <is>
           <t>Columnas 136 (arranque 6.00, sobra 3.00 → se usa en zapatas) + zapatas 29 + VE 22 + VC 18 + cerco 2</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="38">
-      <c r="A20" s="42" t="n">
+    <row r="20" ht="15" customHeight="1" s="43">
+      <c r="A20" s="47" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Varilla Ø1/2" × 9 m</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="47" t="inlineStr">
         <is>
           <t>varilla</t>
         </is>
       </c>
-      <c r="D20" s="62" t="n">
+      <c r="D20" s="67" t="n">
         <v>179</v>
       </c>
-      <c r="E20" s="43" t="n">
+      <c r="E20" s="48" t="n">
         <v>35.96</v>
       </c>
-      <c r="F20" s="43" t="n">
+      <c r="F20" s="48" t="n">
         <v>6436.84</v>
       </c>
-      <c r="G20" s="42" t="inlineStr">
+      <c r="G20" s="47" t="inlineStr">
         <is>
           <t>Estribos columnas 1,342 kg + cerco 177 kg, +5%</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="38">
-      <c r="A21" s="42" t="n">
+    <row r="21" ht="15" customHeight="1" s="43">
+      <c r="A21" s="47" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B21" s="47" t="inlineStr">
         <is>
           <t>Varilla Ø3/8" × 9 m</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C21" s="47" t="inlineStr">
         <is>
           <t>varilla</t>
         </is>
       </c>
-      <c r="D21" s="62" t="n">
+      <c r="D21" s="67" t="n">
         <v>134</v>
       </c>
-      <c r="E21" s="43" t="n">
+      <c r="E21" s="48" t="n">
         <v>20.06</v>
       </c>
-      <c r="F21" s="43" t="n">
+      <c r="F21" s="48" t="n">
         <v>2688.04</v>
       </c>
-      <c r="G21" s="42" t="inlineStr">
+      <c r="G21" s="47" t="inlineStr">
         <is>
           <t>Estribos VE 381 und (4 por varilla) 96 + VC 86 und 13 + montaje 9 + cerco 16</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="38">
-      <c r="A22" s="42" t="n">
+    <row r="22" ht="15" customHeight="1" s="43">
+      <c r="A22" s="47" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B22" s="47" t="inlineStr">
         <is>
           <t>Varilla 6 mm × 9 m</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C22" s="47" t="inlineStr">
         <is>
           <t>varilla</t>
         </is>
       </c>
-      <c r="D22" s="62" t="n">
+      <c r="D22" s="67" t="n">
         <v>15</v>
       </c>
-      <c r="E22" s="43" t="n">
+      <c r="E22" s="48" t="n">
         <v>7.96</v>
       </c>
-      <c r="F22" s="43" t="n">
+      <c r="F22" s="48" t="n">
         <v>119.4</v>
       </c>
-      <c r="G22" s="42" t="inlineStr">
+      <c r="G22" s="47" t="inlineStr">
         <is>
           <t>Cerco 27 kg</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="38">
-      <c r="A23" s="42" t="n">
+    <row r="23" ht="15" customHeight="1" s="43">
+      <c r="A23" s="47" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B23" s="47" t="inlineStr">
         <is>
           <t>Alambre N°16 (3% del acero)</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C23" s="47" t="inlineStr">
         <is>
           <t>rollo</t>
         </is>
       </c>
-      <c r="D23" s="62" t="n">
+      <c r="D23" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="43" t="n">
+      <c r="E23" s="48" t="n">
         <v>349.9</v>
       </c>
-      <c r="F23" s="43" t="n">
+      <c r="F23" s="48" t="n">
         <v>699.8</v>
       </c>
-      <c r="G23" s="42" t="inlineStr">
+      <c r="G23" s="47" t="inlineStr">
         <is>
           <t>176 kg</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="38">
-      <c r="A24" s="51" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="43">
+      <c r="A24" s="56" t="inlineStr">
         <is>
           <t>D. ENCOFRADO Y OTROS</t>
         </is>
       </c>
-      <c r="B24" s="52" t="n"/>
-      <c r="C24" s="52" t="n"/>
-      <c r="D24" s="52" t="n"/>
-      <c r="E24" s="52" t="n"/>
-      <c r="F24" s="52" t="n"/>
-      <c r="G24" s="52" t="n"/>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="38">
-      <c r="A25" s="42" t="n">
+      <c r="B24" s="57" t="n"/>
+      <c r="C24" s="57" t="n"/>
+      <c r="D24" s="57" t="n"/>
+      <c r="E24" s="57" t="n"/>
+      <c r="F24" s="57" t="n"/>
+      <c r="G24" s="57" t="n"/>
+    </row>
+    <row r="25" ht="15" customHeight="1" s="43">
+      <c r="A25" s="47" t="n">
         <v>17</v>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B25" s="47" t="inlineStr">
         <is>
           <t>Alambre N°8 (encofrado)</t>
         </is>
       </c>
-      <c r="C25" s="42" t="inlineStr">
+      <c r="C25" s="47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D25" s="62" t="n">
+      <c r="D25" s="67" t="n">
         <v>58</v>
       </c>
-      <c r="E25" s="43" t="n">
+      <c r="E25" s="48" t="n">
         <v>6.5</v>
       </c>
-      <c r="F25" s="43" t="n">
+      <c r="F25" s="48" t="n">
         <v>377</v>
       </c>
-      <c r="G25" s="42" t="inlineStr">
+      <c r="G25" s="47" t="inlineStr">
         <is>
           <t>0.25 kg/m² × 231 m²</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="38">
-      <c r="A26" s="42" t="n">
+    <row r="26" ht="15" customHeight="1" s="43">
+      <c r="A26" s="47" t="n">
         <v>18</v>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B26" s="47" t="inlineStr">
         <is>
           <t>Clavos</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C26" s="47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D26" s="62" t="n">
+      <c r="D26" s="67" t="n">
         <v>35</v>
       </c>
-      <c r="E26" s="43" t="n">
+      <c r="E26" s="48" t="n">
         <v>7.5</v>
       </c>
-      <c r="F26" s="43" t="n">
+      <c r="F26" s="48" t="n">
         <v>262.5</v>
       </c>
-      <c r="G26" s="42" t="inlineStr">
+      <c r="G26" s="47" t="inlineStr">
         <is>
           <t>0.15 kg/m² × 231 m²</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="38">
-      <c r="A27" s="42" t="n">
+    <row r="27" ht="15" customHeight="1" s="43">
+      <c r="A27" s="47" t="n">
         <v>19</v>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B27" s="47" t="inlineStr">
         <is>
           <t>Ladrillo KK PORTANTE - linderos A y C (+5%)</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C27" s="47" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D27" s="62" t="n">
+      <c r="D27" s="67" t="n">
         <v>2150</v>
       </c>
-      <c r="E27" s="43" t="n">
+      <c r="E27" s="48" t="n">
         <v>1.6</v>
       </c>
-      <c r="F27" s="43" t="n">
+      <c r="F27" s="48" t="n">
         <v>3440</v>
       </c>
-      <c r="G27" s="42" t="inlineStr">
+      <c r="G27" s="47" t="inlineStr">
         <is>
           <t>52.5 m² × 39 × 1.05. Obligatorio en muro portante zona 4 (E.070)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="38">
-      <c r="A28" s="42" t="n">
+    <row r="28" ht="15" customHeight="1" s="43">
+      <c r="A28" s="47" t="n">
         <v>20</v>
       </c>
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B28" s="47" t="inlineStr">
         <is>
           <t>Ladrillo KK 18 huecos - fondo y cerco (+5%)</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C28" s="47" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D28" s="62" t="n">
+      <c r="D28" s="67" t="n">
         <v>1805</v>
       </c>
-      <c r="E28" s="43" t="n">
+      <c r="E28" s="48" t="n">
         <v>1.14</v>
       </c>
-      <c r="F28" s="43" t="n">
+      <c r="F28" s="48" t="n">
         <v>2057.7</v>
       </c>
-      <c r="G28" s="42" t="inlineStr">
+      <c r="G28" s="47" t="inlineStr">
         <is>
           <t>(14.1 + 30.0) m² × 39 × 1.05</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="38">
-      <c r="A29" s="42" t="n">
+    <row r="29" ht="15" customHeight="1" s="43">
+      <c r="A29" s="47" t="n">
         <v>21</v>
       </c>
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>Tecnopor 4" bajo VE</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
         <is>
           <t>plancha</t>
         </is>
       </c>
-      <c r="D29" s="62" t="n">
+      <c r="D29" s="67" t="n">
         <v>3</v>
       </c>
-      <c r="E29" s="43" t="n">
+      <c r="E29" s="48" t="n">
         <v>55</v>
       </c>
-      <c r="F29" s="43" t="n">
+      <c r="F29" s="48" t="n">
         <v>165</v>
       </c>
-      <c r="G29" s="42" t="inlineStr">
+      <c r="G29" s="47" t="inlineStr">
         <is>
           <t>7.4 m² ÷ 2.88</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="38">
-      <c r="A30" s="42" t="n">
+    <row r="30" ht="15" customHeight="1" s="43">
+      <c r="A30" s="47" t="n">
         <v>22</v>
       </c>
-      <c r="B30" s="42" t="inlineStr">
+      <c r="B30" s="47" t="inlineStr">
         <is>
           <t>Tecnopor 1" para juntas</t>
         </is>
       </c>
-      <c r="C30" s="42" t="inlineStr">
+      <c r="C30" s="47" t="inlineStr">
         <is>
           <t>plancha</t>
         </is>
       </c>
-      <c r="D30" s="62" t="n">
+      <c r="D30" s="67" t="n">
         <v>2</v>
       </c>
-      <c r="E30" s="43" t="n">
+      <c r="E30" s="48" t="n">
         <v>16</v>
       </c>
-      <c r="F30" s="43" t="n">
+      <c r="F30" s="48" t="n">
         <v>32</v>
       </c>
-      <c r="G30" s="42" t="inlineStr">
+      <c r="G30" s="47" t="inlineStr">
         <is>
           <t>13.6 ml × 0.13 ≈ 1.8 m² + cortes</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="38">
-      <c r="A31" s="42" t="n">
+    <row r="31" ht="15" customHeight="1" s="43">
+      <c r="A31" s="47" t="n">
         <v>23</v>
       </c>
-      <c r="B31" s="42" t="inlineStr">
+      <c r="B31" s="47" t="inlineStr">
         <is>
           <t>Epóxico para anclajes</t>
         </is>
       </c>
-      <c r="C31" s="42" t="inlineStr">
+      <c r="C31" s="47" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D31" s="62" t="n">
+      <c r="D31" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="43" t="n">
+      <c r="E31" s="48" t="n">
         <v>120</v>
       </c>
-      <c r="F31" s="43" t="n">
+      <c r="F31" s="48" t="n">
         <v>120</v>
       </c>
-      <c r="G31" s="42" t="inlineStr">
+      <c r="G31" s="47" t="inlineStr">
         <is>
           <t>8 anclajes</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="38">
-      <c r="A32" s="42" t="n">
+    <row r="32" ht="15" customHeight="1" s="43">
+      <c r="A32" s="47" t="n">
         <v>24</v>
       </c>
-      <c r="B32" s="42" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>Impermeabilizante asfáltico (sobrecimiento)</t>
         </is>
       </c>
-      <c r="C32" s="42" t="inlineStr">
+      <c r="C32" s="47" t="inlineStr">
         <is>
           <t>gal</t>
         </is>
       </c>
-      <c r="D32" s="62" t="n">
+      <c r="D32" s="67" t="n">
         <v>4</v>
       </c>
-      <c r="E32" s="43" t="n">
+      <c r="E32" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="F32" s="43" t="n">
+      <c r="F32" s="48" t="n">
         <v>180</v>
       </c>
-      <c r="G32" s="42" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="38">
-      <c r="E33" s="45" t="inlineStr">
+      <c r="G32" s="47" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="43">
+      <c r="E33" s="50" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F33" s="46" t="n">
+      <c r="F33" s="51" t="n">
         <v>53866.39</v>
       </c>
     </row>
@@ -2822,235 +2837,235 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="5" customWidth="1" style="37" min="1" max="1"/>
-    <col width="46" customWidth="1" style="37" min="2" max="2"/>
-    <col width="7" customWidth="1" style="37" min="3" max="3"/>
-    <col width="9" customWidth="1" style="37" min="4" max="4"/>
-    <col width="10" customWidth="1" style="37" min="5" max="5"/>
-    <col width="12" customWidth="1" style="37" min="6" max="6"/>
-    <col width="36" customWidth="1" style="37" min="7" max="7"/>
+    <col width="5" customWidth="1" style="42" min="1" max="1"/>
+    <col width="46" customWidth="1" style="42" min="2" max="2"/>
+    <col width="7" customWidth="1" style="42" min="3" max="3"/>
+    <col width="9" customWidth="1" style="42" min="4" max="4"/>
+    <col width="10" customWidth="1" style="42" min="5" max="5"/>
+    <col width="12" customWidth="1" style="42" min="6" max="6"/>
+    <col width="36" customWidth="1" style="42" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="38">
-      <c r="A1" s="39" t="inlineStr">
+    <row r="1" ht="16.15" customHeight="1" s="43">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>EQUIPOS Y SERVICIOS QUE PAGA EL CLIENTE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="38">
-      <c r="A2" s="40" t="n"/>
-    </row>
-    <row r="4" ht="31.5" customHeight="1" s="38">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="43">
+      <c r="A2" s="45" t="n"/>
+    </row>
+    <row r="4" ht="31.5" customHeight="1" s="43">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>N°</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>Concepto</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>Und</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>P.U. (S/)</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>Parcial (S/)</t>
         </is>
       </c>
-      <c r="G4" s="41" t="inlineStr">
+      <c r="G4" s="46" t="inlineStr">
         <is>
           <t>Nota</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="38">
-      <c r="A5" s="42" t="n">
+    <row r="5" ht="15" customHeight="1" s="43">
+      <c r="A5" s="47" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B5" s="47" t="inlineStr">
         <is>
           <t>Eliminación de desmonte - volquete 18 m³</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C5" s="47" t="inlineStr">
         <is>
           <t>viaje</t>
         </is>
       </c>
-      <c r="D5" s="62" t="n">
+      <c r="D5" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="43" t="n">
+      <c r="E5" s="48" t="n">
         <v>460</v>
       </c>
-      <c r="F5" s="43" t="n">
+      <c r="F5" s="48" t="n">
         <v>2300</v>
       </c>
-      <c r="G5" s="42" t="inlineStr">
+      <c r="G5" s="47" t="inlineStr">
         <is>
           <t>78.5 m³ suelto ÷ 18</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="38">
-      <c r="A6" s="42" t="n">
+    <row r="6" ht="15" customHeight="1" s="43">
+      <c r="A6" s="47" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>Alquiler de apisonador para relleno</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>día</t>
         </is>
       </c>
-      <c r="D6" s="62" t="n">
+      <c r="D6" s="67" t="n">
         <v>9</v>
       </c>
-      <c r="E6" s="43" t="n">
+      <c r="E6" s="48" t="n">
         <v>130</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="48" t="n">
         <v>1170</v>
       </c>
-      <c r="G6" s="42" t="inlineStr">
+      <c r="G6" s="47" t="inlineStr">
         <is>
           <t>70.5 m³ ÷ 8 m³/día</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="38">
-      <c r="A7" s="42" t="n">
+    <row r="7" ht="15" customHeight="1" s="43">
+      <c r="A7" s="47" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>Ensayo de probetas</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="47" t="inlineStr">
         <is>
           <t>juego</t>
         </is>
       </c>
-      <c r="D7" s="62" t="n">
+      <c r="D7" s="67" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="43" t="n">
+      <c r="E7" s="48" t="n">
         <v>75</v>
       </c>
-      <c r="F7" s="43" t="n">
+      <c r="F7" s="48" t="n">
         <v>375</v>
       </c>
-      <c r="G7" s="42" t="inlineStr">
+      <c r="G7" s="47" t="inlineStr">
         <is>
           <t>1 por vaciado</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="38">
-      <c r="A8" s="42" t="n">
+    <row r="8" ht="15" customHeight="1" s="43">
+      <c r="A8" s="47" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Combustible apisonador, trompo y vibrador</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>gal</t>
         </is>
       </c>
-      <c r="D8" s="62" t="n">
+      <c r="D8" s="67" t="n">
         <v>20</v>
       </c>
-      <c r="E8" s="43" t="n">
+      <c r="E8" s="48" t="n">
         <v>20</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="48" t="n">
         <v>400</v>
       </c>
-      <c r="G8" s="42" t="n"/>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="38">
-      <c r="A9" s="42" t="n">
+      <c r="G8" s="47" t="n"/>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="43">
+      <c r="A9" s="47" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="47" t="inlineStr">
         <is>
           <t>Agua para obra</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="47" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D9" s="63" t="n">
+      <c r="D9" s="68" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="53" t="n">
+      <c r="E9" s="58" t="n">
         <v>300</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F9" s="48" t="n">
         <v>300</v>
       </c>
-      <c r="G9" s="42" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="38">
-      <c r="A10" s="42" t="n">
+      <c r="G9" s="47" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="43">
+      <c r="A10" s="47" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="47" t="inlineStr">
         <is>
           <t>Flete de fierro y agregados</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D10" s="63" t="n">
+      <c r="D10" s="68" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="53" t="n">
+      <c r="E10" s="58" t="n">
         <v>300</v>
       </c>
-      <c r="F10" s="43" t="n">
+      <c r="F10" s="48" t="n">
         <v>300</v>
       </c>
-      <c r="G10" s="42" t="inlineStr">
+      <c r="G10" s="47" t="inlineStr">
         <is>
           <t>Negociar flete gratis en pedido grande</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="38">
-      <c r="E11" s="45" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="43">
+      <c r="E11" s="50" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F11" s="46" t="n">
+      <c r="F11" s="51" t="n">
         <v>4845</v>
       </c>
     </row>
@@ -3070,835 +3085,835 @@
   <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="7" customWidth="1" style="37" min="1" max="1"/>
-    <col width="56" customWidth="1" style="37" min="2" max="2"/>
-    <col width="6" customWidth="1" style="37" min="3" max="3"/>
-    <col width="10" customWidth="1" style="37" min="4" max="5"/>
-    <col width="12" customWidth="1" style="37" min="6" max="6"/>
-    <col width="2" customWidth="1" style="37" min="7" max="7"/>
-    <col width="12" customWidth="1" style="37" min="8" max="8"/>
-    <col width="11" customWidth="1" style="37" min="9" max="9"/>
-    <col width="30" customWidth="1" style="37" min="10" max="10"/>
-    <col width="11" customWidth="1" style="37" min="11" max="11"/>
-    <col width="2" customWidth="1" style="37" min="12" max="12"/>
-    <col width="20" customWidth="1" style="37" min="13" max="13"/>
-    <col width="10" customWidth="1" style="37" min="14" max="14"/>
-    <col width="8" customWidth="1" style="37" min="15" max="16"/>
+    <col width="7" customWidth="1" style="42" min="1" max="1"/>
+    <col width="56" customWidth="1" style="42" min="2" max="2"/>
+    <col width="6" customWidth="1" style="42" min="3" max="3"/>
+    <col width="10" customWidth="1" style="42" min="4" max="5"/>
+    <col width="12" customWidth="1" style="42" min="6" max="6"/>
+    <col width="2" customWidth="1" style="42" min="7" max="7"/>
+    <col width="12" customWidth="1" style="42" min="8" max="8"/>
+    <col width="11" customWidth="1" style="42" min="9" max="9"/>
+    <col width="30" customWidth="1" style="42" min="10" max="10"/>
+    <col width="11" customWidth="1" style="42" min="11" max="11"/>
+    <col width="2" customWidth="1" style="42" min="12" max="12"/>
+    <col width="20" customWidth="1" style="42" min="13" max="13"/>
+    <col width="10" customWidth="1" style="42" min="14" max="14"/>
+    <col width="8" customWidth="1" style="42" min="15" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.15" customHeight="1" s="38">
-      <c r="A1" s="39" t="inlineStr">
+    <row r="1" ht="16.15" customHeight="1" s="43">
+      <c r="A1" s="44" t="inlineStr">
         <is>
           <t>MANO DE OBRA "POR UN TANTO" - PRECIO AL CLIENTE</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="38">
-      <c r="A2" s="40" t="inlineStr">
+    <row r="2" ht="15" customHeight="1" s="43">
+      <c r="A2" s="45" t="inlineStr">
         <is>
           <t>Precio por partida (mano de obra por un tanto). La excavación incluye la retroexcavadora y el carguío.</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="38"/>
-    <row r="4" ht="31.5" customHeight="1" s="38">
-      <c r="A4" s="41" t="inlineStr">
+    <row r="3" ht="15" customHeight="1" s="43"/>
+    <row r="4" ht="31.5" customHeight="1" s="43">
+      <c r="A4" s="46" t="inlineStr">
         <is>
           <t>Ítem</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="46" t="inlineStr">
         <is>
           <t>Partida</t>
         </is>
       </c>
-      <c r="C4" s="41" t="inlineStr">
+      <c r="C4" s="46" t="inlineStr">
         <is>
           <t>Und</t>
         </is>
       </c>
-      <c r="D4" s="41" t="inlineStr">
+      <c r="D4" s="46" t="inlineStr">
         <is>
           <t>Metrado</t>
         </is>
       </c>
-      <c r="E4" s="41" t="inlineStr">
+      <c r="E4" s="46" t="inlineStr">
         <is>
           <t>P.U. MO (S/)</t>
         </is>
       </c>
-      <c r="F4" s="41" t="inlineStr">
+      <c r="F4" s="46" t="inlineStr">
         <is>
           <t>Parcial (S/)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="38">
-      <c r="A5" s="42" t="inlineStr">
+    <row r="5" ht="15" customHeight="1" s="43">
+      <c r="A5" s="47" t="inlineStr">
         <is>
           <t>01.01</t>
         </is>
       </c>
-      <c r="B5" s="42" t="inlineStr">
+      <c r="B5" s="47" t="inlineStr">
         <is>
           <t>Limpieza de terreno</t>
         </is>
       </c>
-      <c r="C5" s="42" t="inlineStr">
+      <c r="C5" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D5" s="43" t="n">
+      <c r="D5" s="48" t="n">
         <v>170</v>
       </c>
-      <c r="E5" s="43" t="n">
+      <c r="E5" s="48" t="n">
         <v>2.28</v>
       </c>
-      <c r="F5" s="43" t="n">
+      <c r="F5" s="48" t="n">
         <v>387.6</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="38">
-      <c r="A6" s="42" t="inlineStr">
+    <row r="6" ht="15" customHeight="1" s="43">
+      <c r="A6" s="47" t="inlineStr">
         <is>
           <t>01.02</t>
         </is>
       </c>
-      <c r="B6" s="42" t="inlineStr">
+      <c r="B6" s="47" t="inlineStr">
         <is>
           <t>Trazo, nivelación y replanteo</t>
         </is>
       </c>
-      <c r="C6" s="42" t="inlineStr">
+      <c r="C6" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D6" s="43" t="n">
+      <c r="D6" s="48" t="n">
         <v>170</v>
       </c>
-      <c r="E6" s="43" t="n">
+      <c r="E6" s="48" t="n">
         <v>3.43</v>
       </c>
-      <c r="F6" s="43" t="n">
+      <c r="F6" s="48" t="n">
         <v>583.1</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="38">
-      <c r="A7" s="42" t="inlineStr">
+    <row r="7" ht="15" customHeight="1" s="43">
+      <c r="A7" s="47" t="inlineStr">
         <is>
           <t>02.01</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
+      <c r="B7" s="47" t="inlineStr">
         <is>
           <t>Excavación con retroexcavadora (zapatas + zanjas) y carguío</t>
         </is>
       </c>
-      <c r="C7" s="42" t="inlineStr">
+      <c r="C7" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D7" s="43" t="n">
+      <c r="D7" s="48" t="n">
         <v>120</v>
       </c>
-      <c r="E7" s="43" t="n">
+      <c r="E7" s="48" t="n">
         <v>36.55</v>
       </c>
-      <c r="F7" s="43" t="n">
+      <c r="F7" s="48" t="n">
         <v>4386</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="38">
-      <c r="A8" s="42" t="inlineStr">
+    <row r="8" ht="15" customHeight="1" s="43">
+      <c r="A8" s="47" t="inlineStr">
         <is>
           <t>02.02</t>
         </is>
       </c>
-      <c r="B8" s="42" t="inlineStr">
+      <c r="B8" s="47" t="inlineStr">
         <is>
           <t>Perfilado y nivelación de fondos</t>
         </is>
       </c>
-      <c r="C8" s="42" t="inlineStr">
+      <c r="C8" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D8" s="53" t="n">
+      <c r="D8" s="58" t="n">
         <v>75.2</v>
       </c>
-      <c r="E8" s="43" t="n">
+      <c r="E8" s="48" t="n">
         <v>6.85</v>
       </c>
-      <c r="F8" s="43" t="n">
+      <c r="F8" s="48" t="n">
         <v>515.12</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="38">
-      <c r="A9" s="42" t="inlineStr">
+    <row r="9" ht="15" customHeight="1" s="43">
+      <c r="A9" s="47" t="inlineStr">
         <is>
           <t>02.03</t>
         </is>
       </c>
-      <c r="B9" s="42" t="inlineStr">
+      <c r="B9" s="47" t="inlineStr">
         <is>
           <t>Excavación manual cerco</t>
         </is>
       </c>
-      <c r="C9" s="42" t="inlineStr">
+      <c r="C9" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D9" s="43" t="n">
+      <c r="D9" s="48" t="n">
         <v>13.3</v>
       </c>
-      <c r="E9" s="43" t="n">
+      <c r="E9" s="48" t="n">
         <v>51.39</v>
       </c>
-      <c r="F9" s="43" t="n">
+      <c r="F9" s="48" t="n">
         <v>683.487</v>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="38">
-      <c r="A10" s="42" t="inlineStr">
+    <row r="10" ht="15" customHeight="1" s="43">
+      <c r="A10" s="47" t="inlineStr">
         <is>
           <t>02.04</t>
         </is>
       </c>
-      <c r="B10" s="42" t="inlineStr">
+      <c r="B10" s="47" t="inlineStr">
         <is>
           <t>Relleno compactado con material propio</t>
         </is>
       </c>
-      <c r="C10" s="42" t="inlineStr">
+      <c r="C10" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D10" s="43" t="n">
+      <c r="D10" s="48" t="n">
         <v>70.5</v>
       </c>
-      <c r="E10" s="43" t="n">
+      <c r="E10" s="48" t="n">
         <v>34.26</v>
       </c>
-      <c r="F10" s="43" t="n">
+      <c r="F10" s="48" t="n">
         <v>2415.33</v>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="38">
-      <c r="A11" s="42" t="inlineStr">
+    <row r="11" ht="15" customHeight="1" s="43">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>03.01</t>
         </is>
       </c>
-      <c r="B11" s="42" t="inlineStr">
+      <c r="B11" s="47" t="inlineStr">
         <is>
           <t>Solado</t>
         </is>
       </c>
-      <c r="C11" s="42" t="inlineStr">
+      <c r="C11" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D11" s="43" t="n">
+      <c r="D11" s="48" t="n">
         <v>50</v>
       </c>
-      <c r="E11" s="43" t="n">
+      <c r="E11" s="48" t="n">
         <v>17.13</v>
       </c>
-      <c r="F11" s="43" t="n">
+      <c r="F11" s="48" t="n">
         <v>856.5</v>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="38">
-      <c r="A12" s="42" t="inlineStr">
+    <row r="12" ht="15" customHeight="1" s="43">
+      <c r="A12" s="47" t="inlineStr">
         <is>
           <t>03.02</t>
         </is>
       </c>
-      <c r="B12" s="42" t="inlineStr">
+      <c r="B12" s="47" t="inlineStr">
         <is>
           <t>Cimiento corrido ciclópeo cerco</t>
         </is>
       </c>
-      <c r="C12" s="42" t="inlineStr">
+      <c r="C12" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D12" s="43" t="n">
+      <c r="D12" s="48" t="n">
         <v>2.2</v>
       </c>
-      <c r="E12" s="43" t="n">
+      <c r="E12" s="48" t="n">
         <v>102.79</v>
       </c>
-      <c r="F12" s="43" t="n">
+      <c r="F12" s="48" t="n">
         <v>226.138</v>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="38">
-      <c r="A13" s="42" t="inlineStr">
+    <row r="13" ht="15" customHeight="1" s="43">
+      <c r="A13" s="47" t="inlineStr">
         <is>
           <t>03.03</t>
         </is>
       </c>
-      <c r="B13" s="42" t="inlineStr">
+      <c r="B13" s="47" t="inlineStr">
         <is>
           <t>Sobrecimiento - vaciado</t>
         </is>
       </c>
-      <c r="C13" s="42" t="inlineStr">
+      <c r="C13" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D13" s="43" t="n">
+      <c r="D13" s="48" t="n">
         <v>5.85</v>
       </c>
-      <c r="E13" s="43" t="n">
+      <c r="E13" s="48" t="n">
         <v>137.05</v>
       </c>
-      <c r="F13" s="43" t="n">
+      <c r="F13" s="48" t="n">
         <v>801.7424999999999</v>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="38">
-      <c r="A14" s="42" t="inlineStr">
+    <row r="14" ht="15" customHeight="1" s="43">
+      <c r="A14" s="47" t="inlineStr">
         <is>
           <t>03.04</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
+      <c r="B14" s="47" t="inlineStr">
         <is>
           <t>Encofrado y desencofrado de sobrecimiento</t>
         </is>
       </c>
-      <c r="C14" s="42" t="inlineStr">
+      <c r="C14" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D14" s="43" t="n">
+      <c r="D14" s="48" t="n">
         <v>78</v>
       </c>
-      <c r="E14" s="43" t="n">
+      <c r="E14" s="48" t="n">
         <v>25.13</v>
       </c>
-      <c r="F14" s="43" t="n">
+      <c r="F14" s="48" t="n">
         <v>1960.14</v>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="38">
-      <c r="A15" s="42" t="inlineStr">
+    <row r="15" ht="15" customHeight="1" s="43">
+      <c r="A15" s="47" t="inlineStr">
         <is>
           <t>04.09a</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="47" t="inlineStr">
         <is>
           <t>Acero zapatas - habilitado y colocado</t>
         </is>
       </c>
-      <c r="C15" s="42" t="inlineStr">
+      <c r="C15" s="47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D15" s="53" t="n">
+      <c r="D15" s="58" t="n">
         <v>823</v>
       </c>
-      <c r="E15" s="43" t="n">
+      <c r="E15" s="48" t="n">
         <v>1.26</v>
       </c>
-      <c r="F15" s="43" t="n">
+      <c r="F15" s="48" t="n">
         <v>1036.98</v>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="38">
-      <c r="A16" s="42" t="inlineStr">
+    <row r="16" ht="15" customHeight="1" s="43">
+      <c r="A16" s="47" t="inlineStr">
         <is>
           <t>04.09b</t>
         </is>
       </c>
-      <c r="B16" s="42" t="inlineStr">
+      <c r="B16" s="47" t="inlineStr">
         <is>
           <t>Acero VE y VC - habilitado y colocado</t>
         </is>
       </c>
-      <c r="C16" s="42" t="inlineStr">
+      <c r="C16" s="47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D16" s="53" t="n">
+      <c r="D16" s="58" t="n">
         <v>2097</v>
       </c>
-      <c r="E16" s="43" t="n">
+      <c r="E16" s="48" t="n">
         <v>1.26</v>
       </c>
-      <c r="F16" s="43" t="n">
+      <c r="F16" s="48" t="n">
         <v>2642.22</v>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1" s="38">
-      <c r="A17" s="42" t="inlineStr">
+    <row r="17" ht="15" customHeight="1" s="43">
+      <c r="A17" s="47" t="inlineStr">
         <is>
           <t>04.03</t>
         </is>
       </c>
-      <c r="B17" s="42" t="inlineStr">
+      <c r="B17" s="47" t="inlineStr">
         <is>
           <t>Encofrado y desencofrado VE y VC</t>
         </is>
       </c>
-      <c r="C17" s="42" t="inlineStr">
+      <c r="C17" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D17" s="53" t="n">
+      <c r="D17" s="58" t="n">
         <v>51.9</v>
       </c>
-      <c r="E17" s="43" t="n">
+      <c r="E17" s="48" t="n">
         <v>28.55</v>
       </c>
-      <c r="F17" s="43" t="n">
+      <c r="F17" s="48" t="n">
         <v>1481.745</v>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="38">
-      <c r="A18" s="42" t="inlineStr">
+    <row r="18" ht="15" customHeight="1" s="43">
+      <c r="A18" s="47" t="inlineStr">
         <is>
           <t>04.04</t>
         </is>
       </c>
-      <c r="B18" s="42" t="inlineStr">
+      <c r="B18" s="47" t="inlineStr">
         <is>
           <t>Colocación de tecnopor bajo VE</t>
         </is>
       </c>
-      <c r="C18" s="42" t="inlineStr">
+      <c r="C18" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D18" s="43" t="n">
+      <c r="D18" s="48" t="n">
         <v>7.4</v>
       </c>
-      <c r="E18" s="43" t="n">
+      <c r="E18" s="48" t="n">
         <v>5.71</v>
       </c>
-      <c r="F18" s="43" t="n">
+      <c r="F18" s="48" t="n">
         <v>42.254</v>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="38">
-      <c r="A19" s="42" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="43">
+      <c r="A19" s="47" t="inlineStr">
         <is>
           <t>04.01</t>
         </is>
       </c>
-      <c r="B19" s="42" t="inlineStr">
+      <c r="B19" s="47" t="inlineStr">
         <is>
           <t>Vaciado y vibrado premezclado - cimentación (37 m³)</t>
         </is>
       </c>
-      <c r="C19" s="42" t="inlineStr">
+      <c r="C19" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D19" s="53" t="n">
+      <c r="D19" s="58" t="n">
         <v>33.6</v>
       </c>
-      <c r="E19" s="43" t="n">
+      <c r="E19" s="48" t="n">
         <v>45.68</v>
       </c>
-      <c r="F19" s="43" t="n">
+      <c r="F19" s="48" t="n">
         <v>1534.848</v>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="38">
-      <c r="A20" s="42" t="inlineStr">
+    <row r="20" ht="15" customHeight="1" s="43">
+      <c r="A20" s="47" t="inlineStr">
         <is>
           <t>04.09c</t>
         </is>
       </c>
-      <c r="B20" s="42" t="inlineStr">
+      <c r="B20" s="47" t="inlineStr">
         <is>
           <t>Acero columnas - habilitado y colocado (estribos densos)</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D20" s="53" t="n">
+      <c r="D20" s="58" t="n">
         <v>2646</v>
       </c>
-      <c r="E20" s="43" t="n">
+      <c r="E20" s="48" t="n">
         <v>1.48</v>
       </c>
-      <c r="F20" s="43" t="n">
+      <c r="F20" s="48" t="n">
         <v>3916.08</v>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="38">
-      <c r="A21" s="42" t="inlineStr">
+    <row r="21" ht="15" customHeight="1" s="43">
+      <c r="A21" s="47" t="inlineStr">
         <is>
           <t>04.07</t>
         </is>
       </c>
-      <c r="B21" s="42" t="inlineStr">
+      <c r="B21" s="47" t="inlineStr">
         <is>
           <t>Encofrado y desencofrado columnas (h = 3.30)</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C21" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D21" s="43" t="n">
+      <c r="D21" s="48" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="E21" s="43" t="n">
+      <c r="E21" s="48" t="n">
         <v>31.98</v>
       </c>
-      <c r="F21" s="43" t="n">
+      <c r="F21" s="48" t="n">
         <v>2529.618</v>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="38">
-      <c r="A22" s="42" t="inlineStr">
+    <row r="22" ht="15" customHeight="1" s="43">
+      <c r="A22" s="47" t="inlineStr">
         <is>
           <t>04.06</t>
         </is>
       </c>
-      <c r="B22" s="42" t="inlineStr">
+      <c r="B22" s="47" t="inlineStr">
         <is>
           <t>Vaciado y vibrado premezclado - columnas + CA (contra muro endentado)</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C22" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D22" s="53" t="n">
+      <c r="D22" s="58" t="n">
         <v>8.9</v>
       </c>
-      <c r="E22" s="43" t="n">
+      <c r="E22" s="48" t="n">
         <v>68.52</v>
       </c>
-      <c r="F22" s="43" t="n">
+      <c r="F22" s="48" t="n">
         <v>609.828</v>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="38">
-      <c r="A23" s="42" t="inlineStr">
+    <row r="23" ht="15" customHeight="1" s="43">
+      <c r="A23" s="47" t="inlineStr">
         <is>
           <t>04.09d</t>
         </is>
       </c>
-      <c r="B23" s="42" t="inlineStr">
+      <c r="B23" s="47" t="inlineStr">
         <is>
           <t>Acero cerco</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C23" s="47" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="D23" s="53" t="n">
+      <c r="D23" s="58" t="n">
         <v>304</v>
       </c>
-      <c r="E23" s="43" t="n">
+      <c r="E23" s="48" t="n">
         <v>1.37</v>
       </c>
-      <c r="F23" s="43" t="n">
+      <c r="F23" s="48" t="n">
         <v>416.48</v>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="38">
-      <c r="A24" s="42" t="inlineStr">
+    <row r="24" ht="15" customHeight="1" s="43">
+      <c r="A24" s="47" t="inlineStr">
         <is>
           <t>04.08b</t>
         </is>
       </c>
-      <c r="B24" s="42" t="inlineStr">
+      <c r="B24" s="47" t="inlineStr">
         <is>
           <t>Encofrado y desencofrado cerco</t>
         </is>
       </c>
-      <c r="C24" s="42" t="inlineStr">
+      <c r="C24" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D24" s="43" t="n">
+      <c r="D24" s="48" t="n">
         <v>21.9</v>
       </c>
-      <c r="E24" s="43" t="n">
+      <c r="E24" s="48" t="n">
         <v>28.55</v>
       </c>
-      <c r="F24" s="43" t="n">
+      <c r="F24" s="48" t="n">
         <v>625.245</v>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="38">
-      <c r="A25" s="42" t="inlineStr">
+    <row r="25" ht="15" customHeight="1" s="43">
+      <c r="A25" s="47" t="inlineStr">
         <is>
           <t>04.08c</t>
         </is>
       </c>
-      <c r="B25" s="42" t="inlineStr">
+      <c r="B25" s="47" t="inlineStr">
         <is>
           <t>Concreto solera cerco (hecho en obra)</t>
         </is>
       </c>
-      <c r="C25" s="42" t="inlineStr">
+      <c r="C25" s="47" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="D25" s="53" t="n">
+      <c r="D25" s="58" t="n">
         <v>0.37</v>
       </c>
-      <c r="E25" s="43" t="n">
+      <c r="E25" s="48" t="n">
         <v>137.05</v>
       </c>
-      <c r="F25" s="43" t="n">
+      <c r="F25" s="48" t="n">
         <v>50.7085</v>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="38">
-      <c r="A26" s="42" t="inlineStr">
+    <row r="26" ht="15" customHeight="1" s="43">
+      <c r="A26" s="47" t="inlineStr">
         <is>
           <t>04.10</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B26" s="47" t="inlineStr">
         <is>
           <t>Anclajes con epóxico</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C26" s="47" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="D26" s="43" t="n">
+      <c r="D26" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="E26" s="43" t="n">
+      <c r="E26" s="48" t="n">
         <v>22.84</v>
       </c>
-      <c r="F26" s="43" t="n">
+      <c r="F26" s="48" t="n">
         <v>182.72</v>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1" s="38">
-      <c r="A27" s="42" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="43">
+      <c r="A27" s="47" t="inlineStr">
         <is>
           <t>05.01</t>
         </is>
       </c>
-      <c r="B27" s="42" t="inlineStr">
+      <c r="B27" s="47" t="inlineStr">
         <is>
           <t>Muro KK de soga - cerco</t>
         </is>
       </c>
-      <c r="C27" s="42" t="inlineStr">
+      <c r="C27" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D27" s="43" t="n">
+      <c r="D27" s="48" t="n">
         <v>29.8</v>
       </c>
-      <c r="E27" s="43" t="n">
+      <c r="E27" s="48" t="n">
         <v>39.97</v>
       </c>
-      <c r="F27" s="43" t="n">
+      <c r="F27" s="48" t="n">
         <v>1191.106</v>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="38">
-      <c r="A28" s="42" t="inlineStr">
+    <row r="28" ht="15" customHeight="1" s="43">
+      <c r="A28" s="47" t="inlineStr">
         <is>
           <t>05.02a</t>
         </is>
       </c>
-      <c r="B28" s="42" t="inlineStr">
+      <c r="B28" s="47" t="inlineStr">
         <is>
           <t>Muro portante KK endentado - linderos (albañilería confinada)</t>
         </is>
       </c>
-      <c r="C28" s="42" t="inlineStr">
+      <c r="C28" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D28" s="43" t="n">
+      <c r="D28" s="48" t="n">
         <v>52.5</v>
       </c>
-      <c r="E28" s="43" t="n">
+      <c r="E28" s="48" t="n">
         <v>45.68</v>
       </c>
-      <c r="F28" s="43" t="n">
+      <c r="F28" s="48" t="n">
         <v>2398.2</v>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="38">
-      <c r="A29" s="42" t="inlineStr">
+    <row r="29" ht="15" customHeight="1" s="43">
+      <c r="A29" s="47" t="inlineStr">
         <is>
           <t>05.02b</t>
         </is>
       </c>
-      <c r="B29" s="42" t="inlineStr">
+      <c r="B29" s="47" t="inlineStr">
         <is>
           <t>Muro KK de soga - fondo (tabique con junta)</t>
         </is>
       </c>
-      <c r="C29" s="42" t="inlineStr">
+      <c r="C29" s="47" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="D29" s="43" t="n">
+      <c r="D29" s="48" t="n">
         <v>14.1</v>
       </c>
-      <c r="E29" s="43" t="n">
+      <c r="E29" s="48" t="n">
         <v>39.97</v>
       </c>
-      <c r="F29" s="43" t="n">
+      <c r="F29" s="48" t="n">
         <v>563.577</v>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1" s="38">
-      <c r="A30" s="42" t="inlineStr">
+    <row r="30" ht="15" customHeight="1" s="43">
+      <c r="A30" s="47" t="inlineStr">
         <is>
           <t>05.03</t>
         </is>
       </c>
-      <c r="B30" s="42" t="inlineStr">
+      <c r="B30" s="47" t="inlineStr">
         <is>
           <t>Junta con tecnopor 1"</t>
         </is>
       </c>
-      <c r="C30" s="42" t="inlineStr">
+      <c r="C30" s="47" t="inlineStr">
         <is>
           <t>ml</t>
         </is>
       </c>
-      <c r="D30" s="43" t="n">
+      <c r="D30" s="48" t="n">
         <v>13.6</v>
       </c>
-      <c r="E30" s="43" t="n">
+      <c r="E30" s="48" t="n">
         <v>9.140000000000001</v>
       </c>
-      <c r="F30" s="43" t="n">
+      <c r="F30" s="48" t="n">
         <v>124.304</v>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1" s="38">
-      <c r="A31" s="42" t="inlineStr">
+    <row r="31" ht="15" customHeight="1" s="43">
+      <c r="A31" s="47" t="inlineStr">
         <is>
           <t>06.01</t>
         </is>
       </c>
-      <c r="B31" s="42" t="inlineStr">
+      <c r="B31" s="47" t="inlineStr">
         <is>
           <t>Curado de concreto (riego diario)</t>
         </is>
       </c>
-      <c r="C31" s="42" t="inlineStr">
+      <c r="C31" s="47" t="inlineStr">
         <is>
           <t>día</t>
         </is>
       </c>
-      <c r="D31" s="53" t="n">
+      <c r="D31" s="58" t="n">
         <v>14</v>
       </c>
-      <c r="E31" s="43" t="n">
+      <c r="E31" s="48" t="n">
         <v>45.68</v>
       </c>
-      <c r="F31" s="43" t="n">
+      <c r="F31" s="48" t="n">
         <v>639.52</v>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="38">
-      <c r="A32" s="42" t="inlineStr">
+    <row r="32" ht="15" customHeight="1" s="43">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t>06.03</t>
         </is>
       </c>
-      <c r="B32" s="42" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>Limpieza final</t>
         </is>
       </c>
-      <c r="C32" s="42" t="inlineStr">
+      <c r="C32" s="47" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D32" s="53" t="n">
+      <c r="D32" s="58" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="43" t="n">
+      <c r="E32" s="48" t="n">
         <v>342.62</v>
       </c>
-      <c r="F32" s="43" t="n">
+      <c r="F32" s="48" t="n">
         <v>342.62</v>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="38">
-      <c r="B33" s="42" t="inlineStr">
+    <row r="33" ht="15" customHeight="1" s="43">
+      <c r="B33" s="47" t="inlineStr">
         <is>
           <t>Dirección técnica y residencia de obra</t>
         </is>
       </c>
-      <c r="C33" s="42" t="inlineStr">
+      <c r="C33" s="47" t="inlineStr">
         <is>
           <t>glb</t>
         </is>
       </c>
-      <c r="D33" s="63" t="n">
+      <c r="D33" s="68" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="43" t="n">
+      <c r="E33" s="48" t="n">
         <v>2855.17</v>
       </c>
-      <c r="F33" s="43" t="n">
+      <c r="F33" s="48" t="n">
         <v>2855.17</v>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="38">
-      <c r="E34" s="45" t="inlineStr">
+    <row r="34" ht="15" customHeight="1" s="43">
+      <c r="E34" s="50" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F34" s="46" t="n">
+      <c r="F34" s="51" t="n">
         <v>35998.381</v>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="38">
-      <c r="E35" s="64" t="inlineStr">
+    <row r="35" ht="15" customHeight="1" s="43">
+      <c r="E35" s="69" t="inlineStr">
         <is>
           <t>A cotizar (redondeado)</t>
         </is>
       </c>
-      <c r="F35" s="65" t="n">
+      <c r="F35" s="70" t="n">
         <v>36000</v>
       </c>
     </row>

</xml_diff>